<commit_message>
Sync visit form catalogs from failure Excel and improve digital workbook.
Enrich missing clients like MOLYMET/PAE from historial, write visits into the existing maestro Excel, and add Resumen plus extra analysis columns.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mantenimiento_wes/FORMULARIO_MANTENCION_WES_DIGITAL.xlsx
+++ b/mantenimiento_wes/FORMULARIO_MANTENCION_WES_DIGITAL.xlsx
@@ -10,14 +10,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ingreso" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formulario Visita" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base1" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base2" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base3" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base 4" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formulario Visita" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base1" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base2" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base3" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base 4" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Datos'!$B$1:$N$2000</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Datos'!$B$1:$U$2000</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -28,7 +29,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,6 +77,23 @@
       <b val="1"/>
       <color rgb="001F4E79"/>
       <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
     </font>
   </fonts>
   <fills count="7">
@@ -230,7 +248,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -268,6 +286,11 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -640,132 +663,121 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Formulario digital WES = espejo del ingreso automatizado del Sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>Formulario digital WES — mantención / actas</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sheet vivo (fuente oficial): https://docs.google.com/spreadsheets/d/1GlRn7QXWEre7ziau29ojR5lTl-bZ8T3mCT3cD93HZgM</t>
+          <t>Este Excel es el maestro local de análisis. El técnico completa el formulario web;</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Catálogos tomados de: G:\Mi unidad\Agente WES\wes-scripts\mantenimiento wes\maestro\analisis_falla_google.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
+          <t>cada visita se agrega sola a la hoja Datos (y también al Registro de fallas en Drive).</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Hojas:</t>
+          <t>Hojas</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Ingreso — igual al Sheet: Cliente, Máquina, Técnico, Fecha, Tipo mtto,</t>
+          <t xml:space="preserve">  • Ingreso — carga manual rápida (celdas amarillas) si no usan el celular.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Tipo falla, Falla específica, solución, observaciones (+ firma/OT).</t>
+          <t xml:space="preserve">  • Datos — historial (compatible con el Sheet Registro de fallas WES).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Máquina y Falla específica se filtran según Cliente y Tipo de falla</t>
+          <t xml:space="preserve">  • Resumen — totales por cliente / tipo de falla / mes.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">    (requiere Excel 365 o Google Sheets para las fórmulas FILTER).</t>
+          <t xml:space="preserve">  • Formulario Visita — checklist CIR/CPA opcional.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Datos — historial local (se llena con registrar_desde_ingreso.py).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Formulario Visita — checklist CIR/CPA del acta (opcional).</t>
+          <t xml:space="preserve">  • Base1 / Base2 / Base3 / Base 4 — catálogos (Cliente→Máquina, Tipo→Falla).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Base1 / Base2 / Base3 / Base 4 — catálogos y filtros (como el Sheet).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
+          <t>Actualizar clientes / máquinas que faltan</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1) Editá Base1 en el Google Sheet «Registro de fallas WES» (o este Excel).</t>
+        </is>
+      </c>
+    </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Flujo recomendado:</t>
+          <t xml:space="preserve">  2) python sincronizar_catalogos_desde_maestro.py --desde-drive</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1) Completar Ingreso (celdas amarillas).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2) python registrar_desde_ingreso.py</t>
+          <t xml:space="preserve">  3) Reiniciá el servidor del formulario (servir_formulario_visita.py).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3) Pedir al agente el correo de cierre.</t>
+          <t>Flujo recomendado en terreno</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  4) Resumen semanal → Drive carpeta mantenimiento wes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20"/>
+          <t xml:space="preserve">  Celular → formulario web → PDF al cliente (acusar recibo) → fila en Datos.</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Sin Google Form. Firma: acta PDF si el cliente la pide; si no, solo digital.</t>
+          <t>Mejorado: 2026-08-12 19:45</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Generado: 2026-08-11 21:48</t>
+          <t>Catálogos sincronizados: 2026-08-12 19:45 desde analisis_falla_google.xlsx · 28 clientes · 159 máquinas · 62 fallas</t>
         </is>
       </c>
     </row>
@@ -793,14 +805,14 @@
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>INGRESO AUTOMATIZADO — Registro de fallas WES</t>
+          <t>INGRESO — Registro de fallas / visitas WES</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Igual que la hoja Ingreso del Google Sheet. Listas en cascada: Cliente→Máquina y Tipo falla→Falla específica. Celdas amarillas = completar.</t>
+          <t>Celdas amarillas = completar. Listas en cascada Cliente→Máquina y Tipo falla→Falla.</t>
         </is>
       </c>
     </row>
@@ -812,7 +824,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="D4" s="21" t="n"/>
@@ -827,7 +839,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>TOBALABA</t>
+          <t>KFC</t>
         </is>
       </c>
       <c r="D6" s="21" t="n"/>
@@ -913,9 +925,9 @@
           <t>solucion</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>Visita preventiva. Se valida conectividad App, enlace CIR y funcionamiento de válvulas CPA. Sin anomalías críticas.</t>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Prueba carga a Excel maestro existente</t>
         </is>
       </c>
       <c r="D18" s="8" t="n"/>
@@ -934,9 +946,9 @@
           <t>Observaciones</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>Demo del formulario vistoso con PDF + Excel.</t>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>cliente que faltaba en catálogo</t>
         </is>
       </c>
       <c r="D20" s="8" t="n"/>
@@ -957,7 +969,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Sí - acta firmada</t>
+          <t>Sí - Anibal</t>
         </is>
       </c>
       <c r="D22" s="21" t="n"/>
@@ -972,7 +984,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>OT-DEMO-FORM-001</t>
+          <t>OT-PAE-001</t>
         </is>
       </c>
       <c r="D24" s="21" t="n"/>
@@ -997,7 +1009,7 @@
     <row r="28">
       <c r="B28" s="13" t="inlineStr">
         <is>
-          <t>Al terminar: 1) revisar listas  2) ejecutar `python registrar_desde_ingreso.py` para volcar a Datos  3) pedir al agente el correo de cierre  4) Sheet vivo: https://docs.google.com/spreadsheets/d/1GlRn7QXWEre7ziau29ojR5lTl-bZ8T3mCT3cD93HZgM</t>
+          <t>Al terminar (modo Excel): python registrar_desde_ingreso.py  ·  En terreno preferí el formulario web (PDF + correo + esta hoja Datos).</t>
         </is>
       </c>
     </row>
@@ -1023,22 +1035,22 @@
   </mergeCells>
   <dataValidations count="8">
     <dataValidation sqref="C4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Elegí un valor de la lista" type="list">
-      <formula1>Base1!$B$2:$B$147</formula1>
+      <formula1>Base1!$B$2:$B$160</formula1>
     </dataValidation>
     <dataValidation sqref="C6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Elegí un valor de la lista" type="list">
-      <formula1>Base2!$B$1:$B$151</formula1>
+      <formula1>Base2!$B$1:$B$300</formula1>
     </dataValidation>
     <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Elegí un valor de la lista" type="list">
-      <formula1>"Maurico Orellana,Anibal Aranda,Jose Otarola,Gabriel Prieto,Mirko Lorca,Cristian Sepulveda,Salvador Cantillana,Jeans Araya"</formula1>
+      <formula1>"Mauricio Orellana,Maurico Orellana,Anibal Aranda,Jose Otarola,Gabriel Prieto,Mirko Lorca,Cristian Sepulveda,Salvador Cantillana,Jeans Araya"</formula1>
     </dataValidation>
     <dataValidation sqref="C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Elegí un valor de la lista" type="list">
       <formula1>"Mtto Correctivo,Mtto Preventivo,Mtto Predictivo,Reubicacion CIR,Instalación Valvula On/Off,Instalación sistema CIR,Instalación sistema CPA"</formula1>
     </dataValidation>
     <dataValidation sqref="C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Elegí un valor de la lista" type="list">
-      <formula1>Base3!$B$2:$B$67</formula1>
+      <formula1>Base3!$B$2:$B$63</formula1>
     </dataValidation>
     <dataValidation sqref="C16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Elegí un valor de la lista" type="list">
-      <formula1>'Base 4'!$B$1:$B$31</formula1>
+      <formula1>'Base 4'!$B$1:$B$80</formula1>
     </dataValidation>
     <dataValidation sqref="C22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Elegí un valor de la lista" type="list">
       <formula1>"Sí - acta firmada,No - solo digital"</formula1>
@@ -1057,7 +1069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:N51"/>
+  <dimension ref="B1:U51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -1067,12 +1079,19 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="36" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1141,6 +1160,41 @@
           <t>Origen</t>
         </is>
       </c>
+      <c r="O1" s="14" t="inlineStr">
+        <is>
+          <t>Email cliente</t>
+        </is>
+      </c>
+      <c r="P1" s="14" t="inlineStr">
+        <is>
+          <t>Recibido por</t>
+        </is>
+      </c>
+      <c r="Q1" s="14" t="inlineStr">
+        <is>
+          <t>Cargo</t>
+        </is>
+      </c>
+      <c r="R1" s="14" t="inlineStr">
+        <is>
+          <t>Comuna</t>
+        </is>
+      </c>
+      <c r="S1" s="14" t="inlineStr">
+        <is>
+          <t>PDF / Drive</t>
+        </is>
+      </c>
+      <c r="T1" s="14" t="inlineStr">
+        <is>
+          <t>Año</t>
+        </is>
+      </c>
+      <c r="U1" s="14" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="B2" s="15" t="inlineStr">
@@ -1206,66 +1260,353 @@
           <t>Formulario web 2026-08-12 19:10</t>
         </is>
       </c>
+      <c r="O2" s="15" t="n"/>
+      <c r="P2" s="15" t="n"/>
+      <c r="Q2" s="15" t="n"/>
+      <c r="R2" s="15" t="n"/>
+      <c r="S2" s="15" t="n"/>
+      <c r="T2" s="15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="U2" s="15" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="3">
-      <c r="B3" s="15" t="n"/>
-      <c r="C3" s="15" t="n"/>
-      <c r="D3" s="15" t="n"/>
-      <c r="E3" s="24" t="n"/>
-      <c r="F3" s="15" t="n"/>
-      <c r="G3" s="15" t="n"/>
-      <c r="H3" s="15" t="n"/>
-      <c r="I3" s="15" t="n"/>
-      <c r="J3" s="15" t="n"/>
-      <c r="K3" s="15" t="n"/>
-      <c r="L3" s="15" t="n"/>
-      <c r="M3" s="15" t="n"/>
-      <c r="N3" s="15" t="n"/>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>CORMUP</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>TOBALABA</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>Anibal Aranda</t>
+        </is>
+      </c>
+      <c r="E3" s="24" t="n">
+        <v>46246</v>
+      </c>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>Mtto Preventivo</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>Auditoría</t>
+        </is>
+      </c>
+      <c r="H3" s="15" t="inlineStr">
+        <is>
+          <t>Validación Data</t>
+        </is>
+      </c>
+      <c r="I3" s="15" t="inlineStr">
+        <is>
+          <t>Prueba real desde cloud: PDF + correo de acusar recibo.</t>
+        </is>
+      </c>
+      <c r="J3" s="15" t="inlineStr">
+        <is>
+          <t>Simulación de recepción por Anibal.</t>
+        </is>
+      </c>
+      <c r="K3" s="15" t="inlineStr">
+        <is>
+          <t>Sí - Anibal Aranda</t>
+        </is>
+      </c>
+      <c r="L3" s="15" t="inlineStr">
+        <is>
+          <t>OT-PRUEBA-CELULAR-001</t>
+        </is>
+      </c>
+      <c r="M3" s="15" t="inlineStr">
+        <is>
+          <t>cerrada</t>
+        </is>
+      </c>
+      <c r="N3" s="15" t="inlineStr">
+        <is>
+          <t>Formulario web 2026-08-12 19:34</t>
+        </is>
+      </c>
+      <c r="O3" s="15" t="n"/>
+      <c r="P3" s="15" t="n"/>
+      <c r="Q3" s="15" t="n"/>
+      <c r="R3" s="15" t="n"/>
+      <c r="S3" s="15" t="n"/>
+      <c r="T3" s="15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="U3" s="15" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="4">
-      <c r="B4" s="15" t="n"/>
-      <c r="C4" s="15" t="n"/>
-      <c r="D4" s="15" t="n"/>
-      <c r="E4" s="24" t="n"/>
-      <c r="F4" s="15" t="n"/>
-      <c r="G4" s="15" t="n"/>
-      <c r="H4" s="15" t="n"/>
-      <c r="I4" s="15" t="n"/>
-      <c r="J4" s="15" t="n"/>
-      <c r="K4" s="15" t="n"/>
-      <c r="L4" s="15" t="n"/>
-      <c r="M4" s="15" t="n"/>
-      <c r="N4" s="15" t="n"/>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>PROVIDENCIA</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>LASTARRIA</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Anibal Aranda</t>
+        </is>
+      </c>
+      <c r="E4" s="24" t="n">
+        <v>46246</v>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>Mtto Correctivo</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>Hídrica</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>Solenoide</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="inlineStr">
+        <is>
+          <t>Ndjsj</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>Nsnsjs</t>
+        </is>
+      </c>
+      <c r="K4" s="15" t="inlineStr">
+        <is>
+          <t>Sí - Anibal</t>
+        </is>
+      </c>
+      <c r="L4" s="15" t="inlineStr">
+        <is>
+          <t>2251</t>
+        </is>
+      </c>
+      <c r="M4" s="15" t="inlineStr">
+        <is>
+          <t>cerrada</t>
+        </is>
+      </c>
+      <c r="N4" s="15" t="inlineStr">
+        <is>
+          <t>Formulario web 2026-08-12 19:38</t>
+        </is>
+      </c>
+      <c r="O4" s="15" t="n"/>
+      <c r="P4" s="15" t="n"/>
+      <c r="Q4" s="15" t="n"/>
+      <c r="R4" s="15" t="n"/>
+      <c r="S4" s="15" t="n"/>
+      <c r="T4" s="15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="U4" s="15" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="5">
-      <c r="B5" s="15" t="n"/>
-      <c r="C5" s="15" t="n"/>
-      <c r="D5" s="15" t="n"/>
-      <c r="E5" s="24" t="n"/>
-      <c r="F5" s="15" t="n"/>
-      <c r="G5" s="15" t="n"/>
-      <c r="H5" s="15" t="n"/>
-      <c r="I5" s="15" t="n"/>
-      <c r="J5" s="15" t="n"/>
-      <c r="K5" s="15" t="n"/>
-      <c r="L5" s="15" t="n"/>
-      <c r="M5" s="15" t="n"/>
-      <c r="N5" s="15" t="n"/>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>CORMUP</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>TOBALABA</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>Anibal Aranda</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="n">
+        <v>46246</v>
+      </c>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>Mtto Preventivo</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>Auditoría</t>
+        </is>
+      </c>
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>Validación Data</t>
+        </is>
+      </c>
+      <c r="I5" s="15" t="inlineStr">
+        <is>
+          <t>Prueba sync a Sheet maestro</t>
+        </is>
+      </c>
+      <c r="J5" s="15" t="inlineStr">
+        <is>
+          <t>desde agente cloud</t>
+        </is>
+      </c>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>Sí - Anibal</t>
+        </is>
+      </c>
+      <c r="L5" s="15" t="inlineStr">
+        <is>
+          <t>OT-SYNC-001</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>cerrada</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>Formulario web 2026-08-12 19:45</t>
+        </is>
+      </c>
+      <c r="O5" s="15" t="inlineStr">
+        <is>
+          <t>anibal.aoperaciones@wes.cl</t>
+        </is>
+      </c>
+      <c r="P5" s="15" t="inlineStr">
+        <is>
+          <t>Anibal</t>
+        </is>
+      </c>
+      <c r="Q5" s="15" t="n"/>
+      <c r="R5" s="15" t="inlineStr">
+        <is>
+          <t>Providencia</t>
+        </is>
+      </c>
+      <c r="S5" s="15" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/test</t>
+        </is>
+      </c>
+      <c r="T5" s="15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="U5" s="15" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="6">
-      <c r="B6" s="15" t="n"/>
-      <c r="C6" s="15" t="n"/>
-      <c r="D6" s="15" t="n"/>
-      <c r="E6" s="24" t="n"/>
-      <c r="F6" s="15" t="n"/>
-      <c r="G6" s="15" t="n"/>
-      <c r="H6" s="15" t="n"/>
-      <c r="I6" s="15" t="n"/>
-      <c r="J6" s="15" t="n"/>
-      <c r="K6" s="15" t="n"/>
-      <c r="L6" s="15" t="n"/>
-      <c r="M6" s="15" t="n"/>
-      <c r="N6" s="15" t="n"/>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>PAE</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>KFC</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>Anibal Aranda</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="n">
+        <v>46246</v>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>Mtto Preventivo</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>Auditoría</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>Validación Data</t>
+        </is>
+      </c>
+      <c r="I6" s="15" t="inlineStr">
+        <is>
+          <t>Prueba carga a Excel maestro existente</t>
+        </is>
+      </c>
+      <c r="J6" s="15" t="inlineStr">
+        <is>
+          <t>cliente que faltaba en catálogo</t>
+        </is>
+      </c>
+      <c r="K6" s="15" t="inlineStr">
+        <is>
+          <t>Sí - Anibal</t>
+        </is>
+      </c>
+      <c r="L6" s="15" t="inlineStr">
+        <is>
+          <t>OT-PAE-001</t>
+        </is>
+      </c>
+      <c r="M6" s="15" t="inlineStr">
+        <is>
+          <t>cerrada</t>
+        </is>
+      </c>
+      <c r="N6" s="15" t="inlineStr">
+        <is>
+          <t>Formulario web 2026-08-12 19:46</t>
+        </is>
+      </c>
+      <c r="O6" s="15" t="inlineStr">
+        <is>
+          <t>anibal.aoperaciones@wes.cl</t>
+        </is>
+      </c>
+      <c r="P6" s="15" t="inlineStr">
+        <is>
+          <t>Anibal</t>
+        </is>
+      </c>
+      <c r="Q6" s="15" t="n"/>
+      <c r="R6" s="15" t="inlineStr">
+        <is>
+          <t>Santiago</t>
+        </is>
+      </c>
+      <c r="S6" s="15" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/demo</t>
+        </is>
+      </c>
+      <c r="T6" s="15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="U6" s="15" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="15" t="n"/>
@@ -1281,6 +1622,13 @@
       <c r="L7" s="15" t="n"/>
       <c r="M7" s="15" t="n"/>
       <c r="N7" s="15" t="n"/>
+      <c r="O7" s="15" t="n"/>
+      <c r="P7" s="15" t="n"/>
+      <c r="Q7" s="15" t="n"/>
+      <c r="R7" s="15" t="n"/>
+      <c r="S7" s="15" t="n"/>
+      <c r="T7" s="15" t="n"/>
+      <c r="U7" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="15" t="n"/>
@@ -1296,6 +1644,13 @@
       <c r="L8" s="15" t="n"/>
       <c r="M8" s="15" t="n"/>
       <c r="N8" s="15" t="n"/>
+      <c r="O8" s="15" t="n"/>
+      <c r="P8" s="15" t="n"/>
+      <c r="Q8" s="15" t="n"/>
+      <c r="R8" s="15" t="n"/>
+      <c r="S8" s="15" t="n"/>
+      <c r="T8" s="15" t="n"/>
+      <c r="U8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="15" t="n"/>
@@ -1311,6 +1666,13 @@
       <c r="L9" s="15" t="n"/>
       <c r="M9" s="15" t="n"/>
       <c r="N9" s="15" t="n"/>
+      <c r="O9" s="15" t="n"/>
+      <c r="P9" s="15" t="n"/>
+      <c r="Q9" s="15" t="n"/>
+      <c r="R9" s="15" t="n"/>
+      <c r="S9" s="15" t="n"/>
+      <c r="T9" s="15" t="n"/>
+      <c r="U9" s="15" t="n"/>
     </row>
     <row r="10">
       <c r="B10" s="15" t="n"/>
@@ -1326,6 +1688,13 @@
       <c r="L10" s="15" t="n"/>
       <c r="M10" s="15" t="n"/>
       <c r="N10" s="15" t="n"/>
+      <c r="O10" s="15" t="n"/>
+      <c r="P10" s="15" t="n"/>
+      <c r="Q10" s="15" t="n"/>
+      <c r="R10" s="15" t="n"/>
+      <c r="S10" s="15" t="n"/>
+      <c r="T10" s="15" t="n"/>
+      <c r="U10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="15" t="n"/>
@@ -1341,6 +1710,13 @@
       <c r="L11" s="15" t="n"/>
       <c r="M11" s="15" t="n"/>
       <c r="N11" s="15" t="n"/>
+      <c r="O11" s="15" t="n"/>
+      <c r="P11" s="15" t="n"/>
+      <c r="Q11" s="15" t="n"/>
+      <c r="R11" s="15" t="n"/>
+      <c r="S11" s="15" t="n"/>
+      <c r="T11" s="15" t="n"/>
+      <c r="U11" s="15" t="n"/>
     </row>
     <row r="12">
       <c r="B12" s="15" t="n"/>
@@ -1356,6 +1732,13 @@
       <c r="L12" s="15" t="n"/>
       <c r="M12" s="15" t="n"/>
       <c r="N12" s="15" t="n"/>
+      <c r="O12" s="15" t="n"/>
+      <c r="P12" s="15" t="n"/>
+      <c r="Q12" s="15" t="n"/>
+      <c r="R12" s="15" t="n"/>
+      <c r="S12" s="15" t="n"/>
+      <c r="T12" s="15" t="n"/>
+      <c r="U12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="15" t="n"/>
@@ -1371,6 +1754,13 @@
       <c r="L13" s="15" t="n"/>
       <c r="M13" s="15" t="n"/>
       <c r="N13" s="15" t="n"/>
+      <c r="O13" s="15" t="n"/>
+      <c r="P13" s="15" t="n"/>
+      <c r="Q13" s="15" t="n"/>
+      <c r="R13" s="15" t="n"/>
+      <c r="S13" s="15" t="n"/>
+      <c r="T13" s="15" t="n"/>
+      <c r="U13" s="15" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="15" t="n"/>
@@ -1386,6 +1776,13 @@
       <c r="L14" s="15" t="n"/>
       <c r="M14" s="15" t="n"/>
       <c r="N14" s="15" t="n"/>
+      <c r="O14" s="15" t="n"/>
+      <c r="P14" s="15" t="n"/>
+      <c r="Q14" s="15" t="n"/>
+      <c r="R14" s="15" t="n"/>
+      <c r="S14" s="15" t="n"/>
+      <c r="T14" s="15" t="n"/>
+      <c r="U14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="15" t="n"/>
@@ -1401,6 +1798,13 @@
       <c r="L15" s="15" t="n"/>
       <c r="M15" s="15" t="n"/>
       <c r="N15" s="15" t="n"/>
+      <c r="O15" s="15" t="n"/>
+      <c r="P15" s="15" t="n"/>
+      <c r="Q15" s="15" t="n"/>
+      <c r="R15" s="15" t="n"/>
+      <c r="S15" s="15" t="n"/>
+      <c r="T15" s="15" t="n"/>
+      <c r="U15" s="15" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="15" t="n"/>
@@ -1416,6 +1820,13 @@
       <c r="L16" s="15" t="n"/>
       <c r="M16" s="15" t="n"/>
       <c r="N16" s="15" t="n"/>
+      <c r="O16" s="15" t="n"/>
+      <c r="P16" s="15" t="n"/>
+      <c r="Q16" s="15" t="n"/>
+      <c r="R16" s="15" t="n"/>
+      <c r="S16" s="15" t="n"/>
+      <c r="T16" s="15" t="n"/>
+      <c r="U16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="B17" s="15" t="n"/>
@@ -1431,6 +1842,13 @@
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
       <c r="N17" s="15" t="n"/>
+      <c r="O17" s="15" t="n"/>
+      <c r="P17" s="15" t="n"/>
+      <c r="Q17" s="15" t="n"/>
+      <c r="R17" s="15" t="n"/>
+      <c r="S17" s="15" t="n"/>
+      <c r="T17" s="15" t="n"/>
+      <c r="U17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="15" t="n"/>
@@ -1446,6 +1864,13 @@
       <c r="L18" s="15" t="n"/>
       <c r="M18" s="15" t="n"/>
       <c r="N18" s="15" t="n"/>
+      <c r="O18" s="15" t="n"/>
+      <c r="P18" s="15" t="n"/>
+      <c r="Q18" s="15" t="n"/>
+      <c r="R18" s="15" t="n"/>
+      <c r="S18" s="15" t="n"/>
+      <c r="T18" s="15" t="n"/>
+      <c r="U18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="15" t="n"/>
@@ -1461,6 +1886,13 @@
       <c r="L19" s="15" t="n"/>
       <c r="M19" s="15" t="n"/>
       <c r="N19" s="15" t="n"/>
+      <c r="O19" s="15" t="n"/>
+      <c r="P19" s="15" t="n"/>
+      <c r="Q19" s="15" t="n"/>
+      <c r="R19" s="15" t="n"/>
+      <c r="S19" s="15" t="n"/>
+      <c r="T19" s="15" t="n"/>
+      <c r="U19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="15" t="n"/>
@@ -1476,6 +1908,13 @@
       <c r="L20" s="15" t="n"/>
       <c r="M20" s="15" t="n"/>
       <c r="N20" s="15" t="n"/>
+      <c r="O20" s="15" t="n"/>
+      <c r="P20" s="15" t="n"/>
+      <c r="Q20" s="15" t="n"/>
+      <c r="R20" s="15" t="n"/>
+      <c r="S20" s="15" t="n"/>
+      <c r="T20" s="15" t="n"/>
+      <c r="U20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="15" t="n"/>
@@ -1491,6 +1930,13 @@
       <c r="L21" s="15" t="n"/>
       <c r="M21" s="15" t="n"/>
       <c r="N21" s="15" t="n"/>
+      <c r="O21" s="15" t="n"/>
+      <c r="P21" s="15" t="n"/>
+      <c r="Q21" s="15" t="n"/>
+      <c r="R21" s="15" t="n"/>
+      <c r="S21" s="15" t="n"/>
+      <c r="T21" s="15" t="n"/>
+      <c r="U21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="15" t="n"/>
@@ -1506,6 +1952,13 @@
       <c r="L22" s="15" t="n"/>
       <c r="M22" s="15" t="n"/>
       <c r="N22" s="15" t="n"/>
+      <c r="O22" s="15" t="n"/>
+      <c r="P22" s="15" t="n"/>
+      <c r="Q22" s="15" t="n"/>
+      <c r="R22" s="15" t="n"/>
+      <c r="S22" s="15" t="n"/>
+      <c r="T22" s="15" t="n"/>
+      <c r="U22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="15" t="n"/>
@@ -1521,6 +1974,13 @@
       <c r="L23" s="15" t="n"/>
       <c r="M23" s="15" t="n"/>
       <c r="N23" s="15" t="n"/>
+      <c r="O23" s="15" t="n"/>
+      <c r="P23" s="15" t="n"/>
+      <c r="Q23" s="15" t="n"/>
+      <c r="R23" s="15" t="n"/>
+      <c r="S23" s="15" t="n"/>
+      <c r="T23" s="15" t="n"/>
+      <c r="U23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="15" t="n"/>
@@ -1536,6 +1996,13 @@
       <c r="L24" s="15" t="n"/>
       <c r="M24" s="15" t="n"/>
       <c r="N24" s="15" t="n"/>
+      <c r="O24" s="15" t="n"/>
+      <c r="P24" s="15" t="n"/>
+      <c r="Q24" s="15" t="n"/>
+      <c r="R24" s="15" t="n"/>
+      <c r="S24" s="15" t="n"/>
+      <c r="T24" s="15" t="n"/>
+      <c r="U24" s="15" t="n"/>
     </row>
     <row r="25">
       <c r="B25" s="15" t="n"/>
@@ -1551,6 +2018,13 @@
       <c r="L25" s="15" t="n"/>
       <c r="M25" s="15" t="n"/>
       <c r="N25" s="15" t="n"/>
+      <c r="O25" s="15" t="n"/>
+      <c r="P25" s="15" t="n"/>
+      <c r="Q25" s="15" t="n"/>
+      <c r="R25" s="15" t="n"/>
+      <c r="S25" s="15" t="n"/>
+      <c r="T25" s="15" t="n"/>
+      <c r="U25" s="15" t="n"/>
     </row>
     <row r="26">
       <c r="B26" s="15" t="n"/>
@@ -1566,6 +2040,13 @@
       <c r="L26" s="15" t="n"/>
       <c r="M26" s="15" t="n"/>
       <c r="N26" s="15" t="n"/>
+      <c r="O26" s="15" t="n"/>
+      <c r="P26" s="15" t="n"/>
+      <c r="Q26" s="15" t="n"/>
+      <c r="R26" s="15" t="n"/>
+      <c r="S26" s="15" t="n"/>
+      <c r="T26" s="15" t="n"/>
+      <c r="U26" s="15" t="n"/>
     </row>
     <row r="27">
       <c r="B27" s="15" t="n"/>
@@ -1581,6 +2062,13 @@
       <c r="L27" s="15" t="n"/>
       <c r="M27" s="15" t="n"/>
       <c r="N27" s="15" t="n"/>
+      <c r="O27" s="15" t="n"/>
+      <c r="P27" s="15" t="n"/>
+      <c r="Q27" s="15" t="n"/>
+      <c r="R27" s="15" t="n"/>
+      <c r="S27" s="15" t="n"/>
+      <c r="T27" s="15" t="n"/>
+      <c r="U27" s="15" t="n"/>
     </row>
     <row r="28">
       <c r="B28" s="15" t="n"/>
@@ -1596,6 +2084,13 @@
       <c r="L28" s="15" t="n"/>
       <c r="M28" s="15" t="n"/>
       <c r="N28" s="15" t="n"/>
+      <c r="O28" s="15" t="n"/>
+      <c r="P28" s="15" t="n"/>
+      <c r="Q28" s="15" t="n"/>
+      <c r="R28" s="15" t="n"/>
+      <c r="S28" s="15" t="n"/>
+      <c r="T28" s="15" t="n"/>
+      <c r="U28" s="15" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="15" t="n"/>
@@ -1611,6 +2106,13 @@
       <c r="L29" s="15" t="n"/>
       <c r="M29" s="15" t="n"/>
       <c r="N29" s="15" t="n"/>
+      <c r="O29" s="15" t="n"/>
+      <c r="P29" s="15" t="n"/>
+      <c r="Q29" s="15" t="n"/>
+      <c r="R29" s="15" t="n"/>
+      <c r="S29" s="15" t="n"/>
+      <c r="T29" s="15" t="n"/>
+      <c r="U29" s="15" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="15" t="n"/>
@@ -1626,6 +2128,13 @@
       <c r="L30" s="15" t="n"/>
       <c r="M30" s="15" t="n"/>
       <c r="N30" s="15" t="n"/>
+      <c r="O30" s="15" t="n"/>
+      <c r="P30" s="15" t="n"/>
+      <c r="Q30" s="15" t="n"/>
+      <c r="R30" s="15" t="n"/>
+      <c r="S30" s="15" t="n"/>
+      <c r="T30" s="15" t="n"/>
+      <c r="U30" s="15" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="15" t="n"/>
@@ -1641,6 +2150,13 @@
       <c r="L31" s="15" t="n"/>
       <c r="M31" s="15" t="n"/>
       <c r="N31" s="15" t="n"/>
+      <c r="O31" s="15" t="n"/>
+      <c r="P31" s="15" t="n"/>
+      <c r="Q31" s="15" t="n"/>
+      <c r="R31" s="15" t="n"/>
+      <c r="S31" s="15" t="n"/>
+      <c r="T31" s="15" t="n"/>
+      <c r="U31" s="15" t="n"/>
     </row>
     <row r="32">
       <c r="B32" s="15" t="n"/>
@@ -1656,6 +2172,13 @@
       <c r="L32" s="15" t="n"/>
       <c r="M32" s="15" t="n"/>
       <c r="N32" s="15" t="n"/>
+      <c r="O32" s="15" t="n"/>
+      <c r="P32" s="15" t="n"/>
+      <c r="Q32" s="15" t="n"/>
+      <c r="R32" s="15" t="n"/>
+      <c r="S32" s="15" t="n"/>
+      <c r="T32" s="15" t="n"/>
+      <c r="U32" s="15" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="15" t="n"/>
@@ -1671,6 +2194,13 @@
       <c r="L33" s="15" t="n"/>
       <c r="M33" s="15" t="n"/>
       <c r="N33" s="15" t="n"/>
+      <c r="O33" s="15" t="n"/>
+      <c r="P33" s="15" t="n"/>
+      <c r="Q33" s="15" t="n"/>
+      <c r="R33" s="15" t="n"/>
+      <c r="S33" s="15" t="n"/>
+      <c r="T33" s="15" t="n"/>
+      <c r="U33" s="15" t="n"/>
     </row>
     <row r="34">
       <c r="B34" s="15" t="n"/>
@@ -1686,6 +2216,13 @@
       <c r="L34" s="15" t="n"/>
       <c r="M34" s="15" t="n"/>
       <c r="N34" s="15" t="n"/>
+      <c r="O34" s="15" t="n"/>
+      <c r="P34" s="15" t="n"/>
+      <c r="Q34" s="15" t="n"/>
+      <c r="R34" s="15" t="n"/>
+      <c r="S34" s="15" t="n"/>
+      <c r="T34" s="15" t="n"/>
+      <c r="U34" s="15" t="n"/>
     </row>
     <row r="35">
       <c r="B35" s="15" t="n"/>
@@ -1943,12 +2480,66 @@
       <c r="N51" s="15" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:N2000"/>
+  <autoFilter ref="B1:U2000"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Resumen operativo (desde hoja Datos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Total visitas registradas</t>
+        </is>
+      </c>
+      <c r="B3" s="27">
+        <f>COUNTA(Datos!B:B)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Clientes distintos</t>
+        </is>
+      </c>
+      <c r="B4" s="28">
+        <f>IFERROR(SUMPRODUCT((Datos!B2:B2000&lt;&gt;"")/COUNTIF(Datos!B2:B2000,Datos!B2:B2000&amp;"")),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>Tip: filtrá la hoja Datos por Cliente / Año / Mes para el análisis semanal.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2519,26 +3110,26 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C147"/>
+  <dimension ref="B1:C160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="18" t="inlineStr">
+      <c r="B1" s="25" t="inlineStr">
         <is>
           <t>CLIENTE</t>
         </is>
       </c>
-      <c r="C1" s="18" t="inlineStr">
+      <c r="C1" s="25" t="inlineStr">
         <is>
           <t>MAQUINA</t>
         </is>
@@ -2547,780 +3138,780 @@
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>AEB</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ESCUELA VILLA INDEPENDENCIA</t>
+          <t>MATRIZ A.A</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>AEB</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ESCUELA ANDES DEL SUR</t>
+          <t>MATRIZ PRIMER PISO</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>AEB</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ESCUELA PADRE HURTADO</t>
+          <t>MATRIZ RIEGO PLAZA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>AGUNSA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>LICEO MAIPO</t>
+          <t>DEPOSITO</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>AGUNSA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ESCUELA LUIS MATTE LARRAIN</t>
+          <t>MODULO ABC</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>AGUNSA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ESCUELA GABRIELA</t>
+          <t>MODULO D</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>AGUNSA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ESCUELA JUAN MACKENNA</t>
+          <t>MODULO E</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>BOM</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LICEO CHILOE</t>
+          <t>SAN IGNACIO 300</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>BOM</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ESCUELA LOS ANDES</t>
+          <t>SAN IGNACIO 500</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>COMPLEJO EDUCACIONAL CONSOLIDADA</t>
+          <t>CALLE DE SERVICO</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ESCULA NONATO COO</t>
+          <t>CLUB HOUSE</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CENTRO EDUCACIONAL EDUARDO DE LA BARRA</t>
+          <t>EDIFICIO DEPORTIVO</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CARLOS FERNANDEZ PEÑA</t>
+          <t>EDIFIO DEPORTIVO</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>TOBALABA</t>
+          <t>EQUITACION</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ANTONIO HERMIDA FABRES</t>
+          <t>RAIMUNDO TUPPER</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SANTA MARIA</t>
+          <t>COSTANERA</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ESCUELA LUIS ARRIETA CAÑAS</t>
+          <t>ESTANQUE DE REUTILIZACION</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ERASMO ESCALA</t>
+          <t>LAVADO AUTO SERVICIO NORTE</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ALICURA</t>
+          <t>LAVADO AUTO SERVICIO SUR</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>JUAN BAUTISTA PASTENE</t>
+          <t>LAVADO AUTOMATICO NORTE</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MATILDE HUICI NAVAS</t>
+          <t>LAVADO AUTOMATICO SUR</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CENTRO EDUCACIONAL VALLE HERMOSO</t>
+          <t>MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ESCUELA UNIÓN NACIONAL ÁRABE</t>
+          <t>OFICINA ADMIN</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LIKANKURA</t>
+          <t>PRONTO BAÑO</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ESCUELA ESPECIAL PONTÍFICE JUAN PABLO II</t>
+          <t>PRONTO TIENDA</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CDP PUENTE ALTO</t>
+          <t>RIEGO</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>CPF SAN MIGUEL SALA IMPULSION</t>
+          <t>COMPLEJO EDUCACIONAL CONSOLIDADA</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>COLINA 1</t>
+          <t>ESCUELA ANDES DEL SUR</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>COLINA 2 RED SUR</t>
+          <t>ESCUELA GABRIELA</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CPF SAN MIGUEL MATRIZ PRINCIPAL</t>
+          <t>ESCUELA JUAN MACKENNA</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>COLINA 2 REDIMPULSION</t>
+          <t>ESCUELA LOS ANDES</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>CPA OVALO</t>
+          <t>ESCUELA LUIS MATTE LARRAIN</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CPA MODULO</t>
+          <t>ESCUELA PADRE HURTADO</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MONITOREO MATRIZ PRINCIPAL OVALO</t>
+          <t>ESCUELA VILLA INDEPENDENCIA</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MONITOREO MATRIZ PRINCIPAL MODULO</t>
+          <t>ESCULA NONATO COO</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ESFORPEN BOSQUE ADMINISTRACION</t>
+          <t>LICEO CHILOE</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ESFORPEN BOSQUE GENCHI SIMULACION</t>
+          <t>LICEO MAIPO</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ESC. OF CARMEN</t>
+          <t>ALICURA</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ESC. OF ARTEMIO</t>
+          <t>ANTONIO HERMIDA FABRES</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>CARLOS FERNANDEZ PEÑA</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ESTANQUE DE REUTILIZACION</t>
+          <t>CENTRO EDUCACIONAL EDUARDO DE LA BARRA</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LAVADO AUTOMATICO NORTE</t>
+          <t>CENTRO EDUCACIONAL VALLE HERMOSO</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>LAVADO AUTOMATICO SUR</t>
+          <t>ERASMO ESCALA</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>OFICINA ADMIN</t>
+          <t>ESCUELA ESPECIAL PONTÍFICE JUAN PABLO II</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>RIEGO</t>
+          <t>ESCUELA LUIS ARRIETA CAÑAS</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>PRONTO BAÑO</t>
+          <t>ESCUELA UNIÓN NACIONAL ÁRABE</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>PRONTO TIENDA</t>
+          <t>JUAN BAUTISTA PASTENE</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>LAVADO AUTO SERVICIO NORTE</t>
+          <t>LIKANKURA</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>LAVADO AUTO SERVICIO SUR</t>
+          <t>MATILDE HUICI NAVAS</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>COSTANERA</t>
+          <t>SANTA MARIA</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ESTANQUE B</t>
+          <t>TOBALABA</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>CUR</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>TEATRO</t>
+          <t>ANILLO NORTE</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>CUR</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>HIGH SCHOOL</t>
+          <t>ANILLO SUR</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>CUR</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ELEMENTARY</t>
+          <t>BAÑOS</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>CUR</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>POZO PROFUNDO</t>
+          <t>MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ESTANQUE C</t>
+          <t>LO BOZA - EDIFICIO PRINCIPAL CASINO</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="B58" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>CANCHA</t>
+          <t>LO BOZA - LAVADO DE VEHICULOS</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>CONTROL NIDO</t>
+          <t>LO BOZA - POZO DE LAVADO DE VEHICULO</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="B60" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>PISCINA</t>
+          <t>LO BOZA - REUTILIZACION</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="B61" t="inlineStr">
         <is>
-          <t>LO VALLEDOR</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>PUERTA 1</t>
+          <t>LO BOZA - SALA DE IMPULSION</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="B62" t="inlineStr">
         <is>
-          <t>LO VALLEDOR</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>POZO 1</t>
+          <t>OPEN PLAZA - MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="B63" t="inlineStr">
         <is>
-          <t>LO VALLEDOR</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>BARRIO NORTE</t>
+          <t>PRONTO BAÑO</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="B64" t="inlineStr">
         <is>
-          <t>PROVIDENCIA</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>LASTARRIA</t>
+          <t>QUILICURA - CAMARINES</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="B65" t="inlineStr">
         <is>
-          <t>PROVIDENCIA</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>ARTURO ALESSANDRI PALMA</t>
+          <t>QUILICURA - CASINO</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="B66" t="inlineStr">
         <is>
-          <t>PROVIDENCIA</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>CARMELA CARVAJAL</t>
+          <t>QUILICURA - DERCOMAQ</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3923,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>LO BOZA - LAVADO DE VEHICULOS</t>
+          <t>QUILICURA - EDIFICIO JCB</t>
         </is>
       </c>
     </row>
@@ -3344,7 +3935,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>LO BOZA - POZO DE LAVADO DE VEHICULO</t>
+          <t>QUILICURA - LAVADO DE MAQUINA</t>
         </is>
       </c>
     </row>
@@ -3356,7 +3947,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>LO BOZA - REUTILIZACION</t>
+          <t>QUILICURA - MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -3368,511 +3959,511 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>LO BOZA - SALA DE IMPULSION</t>
+          <t>QUILICURA - PRODERCO</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="B71" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>ESTADIO ISRAELITA</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>LO BOZA - EDIFICIO PRINCIPAL CASINO</t>
+          <t>MATRIS CHESTERTON</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="B72" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>ESTADIO ISRAELITA</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>QUILICURA - MATRIZ PRINCIPAL</t>
+          <t>MATRIZ AV LAS CONDES</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="B73" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>QUILICURA - DERCOMAQ</t>
+          <t>ETAPA 1,2,3 Y 4</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="B74" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>QUILICURA - LAVADO DE MAQUINA</t>
+          <t>ETAPA 5</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="B75" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>QUILICURA - CASINO</t>
+          <t>MATRIS ESVAL</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="B76" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>QUILICURA - PRODERCO</t>
+          <t>RIEGO</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="B77" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>QUILICURA - CAMARINES</t>
+          <t>CDP PUENTE ALTO</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="B78" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>QUILICURA - EDIFICIO JCB</t>
+          <t>COLINA 1</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="B79" t="inlineStr">
         <is>
-          <t>RENCA</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>REBECA MATTE BELLO</t>
+          <t>COLINA 2 RED SUR</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="B80" t="inlineStr">
         <is>
-          <t>RENCA</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>JUAN DE ATALA HIRMAS</t>
+          <t>COLINA 2 REDIMPULSION</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="B81" t="inlineStr">
         <is>
-          <t>RENCA</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>CAPITAN JOSÉ LUIS ARANDE</t>
+          <t>CPA MODULO</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="B82" t="inlineStr">
         <is>
-          <t>LAS CONDES</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>FLEMING</t>
+          <t>CPA OVALO</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="B83" t="inlineStr">
         <is>
-          <t>LAS CONDES</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>JUAN PABLO II</t>
+          <t>CPF SAN MIGUEL MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="B84" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>CPF SAN MIGUEL SALA IMPULSION</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="B85" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>AGUA BLANDA</t>
+          <t>ESC. EL BOSQUE ADMINISTRACION</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="B86" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>SALIDA OSMOSIS</t>
+          <t>ESC. EL BOSQUE GENCHI ACADEMIA</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="B87" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>RETORNO OSMOSIS</t>
+          <t>ESC. OF ARTEMIO</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="B88" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>INTERCAMBIADOR 1</t>
+          <t>ESC. OF CARMEN</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="B89" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>INTERCAMBIADOR 2</t>
+          <t>ESCUELA ANDES DEL SUR</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="B90" t="inlineStr">
         <is>
-          <t>AGUNSA</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>DEPOSITO</t>
+          <t>ESFORPEN BOSQUE ADMINISTRACION</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="B91" t="inlineStr">
         <is>
-          <t>AGUNSA</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>MODULO D</t>
+          <t>ESFORPEN BOSQUE GENCHI SIMULACION</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="B92" t="inlineStr">
         <is>
-          <t>AGUNSA</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>MODULO ABC</t>
+          <t>MONITOREO MATRIZ PRINCIPAL MODULO</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="B93" t="inlineStr">
         <is>
-          <t>AGUNSA</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>MODULO E</t>
+          <t>MONITOREO MATRIZ PRINCIPAL OVALO</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="B94" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>CLUB HOUSE</t>
+          <t>AGUA BLANDA</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="B95" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>EDIFIO DEPORTIVO</t>
+          <t>INTERCAMBIADOR 1</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="B96" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>CALLE DE SERVICO</t>
+          <t>INTERCAMBIADOR 2</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="B97" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>RAIMUNDO TUPPER</t>
+          <t>MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="B98" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>EQUITACION</t>
+          <t>RETORNO OSMOSIS</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="B99" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>ESTANQUE CISTERNA</t>
+          <t>SALIDA OSMOSIS</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="B100" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>LA FLORIDA</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>SAN NICOLAS</t>
+          <t>LICEO ALTO CORDILLERA</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="B101" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>LA REINA</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>URETA COX</t>
+          <t>EUGENIO MARIA DE HOSTOS</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>LAS CONDES</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>CASINO</t>
+          <t>FLEMING</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="B103" t="inlineStr">
         <is>
-          <t>LA REINA</t>
+          <t>LAS CONDES</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>EUGENIO MARIA DE HOSTOS</t>
+          <t>JUAN PABLO II</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
-          <t>UDD</t>
+          <t>LAS CONDES</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS EDIFICIO ¨O¨</t>
+          <t>LIKANKURA</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="B105" t="inlineStr">
         <is>
-          <t>UDD</t>
+          <t>LO VALLEDOR</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS HONDURAS</t>
+          <t>BARRIO NORTE</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="B106" t="inlineStr">
         <is>
-          <t>LA FLORIDA</t>
+          <t>LO VALLEDOR</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>LICEO ALTO CORDILLERA</t>
+          <t>POZO 1</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="B107" t="inlineStr">
         <is>
-          <t>ESTADIO ISRAELITA</t>
+          <t>LO VALLEDOR</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATRIZ AV LAS CONDES </t>
+          <t>PUERTA 1</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="B108" t="inlineStr">
         <is>
-          <t>ESTADIO ISRAELITA</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>MATRIS CHESTERTON</t>
+          <t>CASINO</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>MATRIS ESVAL</t>
+          <t>ESTANQUE CISTERNA</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="B110" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>ETAPA 1,2,3 Y 4</t>
+          <t>SAN NICOLAS</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="B111" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>ETAPA 5</t>
+          <t>URETA COX</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="B112" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>RIEGO</t>
+          <t>BAÑO GUARDIAS</t>
         </is>
       </c>
     </row>
@@ -3884,7 +4475,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>ESTANQUE NORTE LOCALES</t>
+          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
         </is>
       </c>
     </row>
@@ -3896,7 +4487,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
+          <t>ESTANQUE NORTE LOCALES</t>
         </is>
       </c>
     </row>
@@ -3908,7 +4499,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>KFC</t>
+          <t>ESTANQUE SUR ABASTECIMIENTO</t>
         </is>
       </c>
     </row>
@@ -3920,7 +4511,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>PIZZA HUT</t>
+          <t>KFC</t>
         </is>
       </c>
     </row>
@@ -3932,86 +4523,86 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ESTANQUE SUR ABASTECIMIENTO</t>
+          <t>PIZZA HUT</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="B118" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>BAÑO GUARDIAS</t>
+          <t>MATRIZ BOULEVARD PASILLO TECNICO</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="B119" t="inlineStr">
         <is>
-          <t>AEB</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>MATRIZ A.A</t>
+          <t>MATRIZ SALIDA DE EMERGENCIA PASILLO N°1 ARROW</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="B120" t="inlineStr">
         <is>
-          <t>AEB</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>MATRIZ PRIMER PISO</t>
+          <t>PLACA BANCARIA</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="B121" t="inlineStr">
         <is>
-          <t>AEB</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>MATRIZ RIEGO PLAZA</t>
+          <t>SALA DE BOMBAS FALABELLA</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="B122" t="inlineStr">
         <is>
-          <t>BOM</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>SAN IGNACIO 500</t>
+          <t>SALA DE BOMBAS RIPLEY</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="B123" t="inlineStr">
         <is>
-          <t>BOM</t>
+          <t>MAQ</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>SAN IGNACIO 300</t>
+          <t>ALIMENTACION DE BAÑOS</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="B124" t="inlineStr">
         <is>
-          <t>CUR</t>
+          <t>MAQ</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -4023,192 +4614,192 @@
     <row r="125">
       <c r="B125" t="inlineStr">
         <is>
-          <t>CUR</t>
+          <t>MAQ</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>BAÑOS</t>
+          <t>RED DE INCENDIO</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="B126" t="inlineStr">
         <is>
-          <t>CUR</t>
+          <t>MOLYMET</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>ANILLO SUR</t>
+          <t>CASA DE CAMBIO</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="B127" t="inlineStr">
         <is>
-          <t>CUR</t>
+          <t>MOLYMET</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>ANILLO NORTE</t>
+          <t>RIEGO</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="B128" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>PLACA BANCARIA</t>
+          <t>CANCHA</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="B129" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS FALABELLA</t>
+          <t>CONTROL NIDO</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="B130" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS RIPLEY</t>
+          <t>ELEMENTARY</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="B131" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>MATRIZ BOULEVARD PASILLO TECNICO</t>
+          <t>ESTANQUE B</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="B132" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>MATRIZ SALIDA DE EMERGENCIA PASILLO N°1 ARROW</t>
+          <t>ESTANQUE C</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="B133" t="inlineStr">
         <is>
-          <t>MAQ</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>HIGH SCHOOL</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="B134" t="inlineStr">
         <is>
-          <t>MAQ</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ALIMENTACION DE BAÑOS</t>
+          <t>PISCINA</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="B135" t="inlineStr">
         <is>
-          <t>MAQ</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>RED DE INCENDIO</t>
+          <t>POZO PROFUNDO</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="B136" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>SANDIA ANTIGUA</t>
+          <t>TEATRO</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="B137" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>DISTRITO DE LUJO</t>
+          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="B138" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>PILETA CASCADA</t>
+          <t>ESTANQUE NORTE LOCALES</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="B139" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>LLENADO DE PILETA</t>
+          <t>KFC</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="B140" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>SANDIA NUEVA</t>
+          <t>PIZZA HUT</t>
         </is>
       </c>
     </row>
@@ -4220,7 +4811,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>BAZAR GOURMET</t>
+          <t>ANDEN 3-4 LOCALES GASTRONOMICOS</t>
         </is>
       </c>
     </row>
@@ -4232,7 +4823,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>DL KENNEDY</t>
+          <t>ANDEN 3-4 MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -4244,7 +4835,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>ANDEN 3-4 MATRIZ PRINCIPAL</t>
+          <t>ANDEN 3-4 RESTAURANTE</t>
         </is>
       </c>
     </row>
@@ -4256,7 +4847,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>ANDEN 3-4 LOCALES GASTRONOMICOS</t>
+          <t>BAZAR GOURMET</t>
         </is>
       </c>
     </row>
@@ -4268,7 +4859,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>ANDEN 3-4 RESTAURANTE</t>
+          <t>BAÑO DAMAS</t>
         </is>
       </c>
     </row>
@@ -4280,7 +4871,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>BAÑO DAMAS</t>
+          <t>BAÑO VARONES</t>
         </is>
       </c>
     </row>
@@ -4292,7 +4883,163 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>BAÑO VARONES</t>
+          <t>DISTRITO DE LUJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>PAK</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>DL KENNEDY</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>PAK</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>LLENADO DE PILETA</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>PAK</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>PILETA CASCADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>PAK</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>SANDIA ANTIGUA</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>PAK</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>SANDIA NUEVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>PROVIDENCIA</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>ARTURO ALESSANDRI PALMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>PROVIDENCIA</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>CARMELA CARVAJAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>PROVIDENCIA</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>LASTARRIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>CAPITAN JOSÉ LUIS ARANDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>JUAN DE ATALA HIRMAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>REBECA MATTE BELLO</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>UDD</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>SALA DE BOMBAS EDIFICIO ¨O¨</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>UDD</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>SALA DE BOMBAS HONDURAS</t>
         </is>
       </c>
     </row>
@@ -4301,7 +5048,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4316,7 +5063,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="20">
-        <f>IFERROR(FILTER(Base1!B2:C147,Base1!B2:B147=Ingreso!C4),"")</f>
+        <f>IFERROR(FILTER(Base1!B2:C160,Base1!B2:B160=Ingreso!C4),"")</f>
         <v/>
       </c>
     </row>
@@ -4325,13 +5072,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C67"/>
+  <dimension ref="B1:C63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -4339,12 +5086,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="18" t="inlineStr">
+      <c r="B1" s="25" t="inlineStr">
         <is>
           <t>Tipo de falla</t>
         </is>
       </c>
-      <c r="C1" s="18" t="inlineStr">
+      <c r="C1" s="25" t="inlineStr">
         <is>
           <t>Falla Específica</t>
         </is>
@@ -4353,216 +5100,216 @@
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Auditoría</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Cortocircuito</t>
+          <t>Toma de Lectura Inicial</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Auditoría</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Empalme electrico</t>
+          <t>Toma de Lectura Final</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Auditoría</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fusible Cortado</t>
+          <t>Validación Data</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Comunicación</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Falla Fuente switching</t>
+          <t>Max 232</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Comunicación</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Intervencion de terceros</t>
+          <t>Placa Conversor RS232 mala</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Comunicación</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Cargador Solar</t>
+          <t>Conector DB9</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Comunicación</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Bateria Descargada</t>
+          <t>Router</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>Electrónica</t>
+          <t>Comunicación</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Componente dañado</t>
+          <t>Amplimax</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>Electrónica</t>
+          <t>Comunicación</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Ruido</t>
+          <t>Sim</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>Electrónica</t>
+          <t>Comunicación</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Placa Pegada</t>
+          <t>Conector tx rx</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>Electrónica</t>
+          <t>Comunicación</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Reloj Malo</t>
+          <t>ID Erróneo</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
-          <t>Electrónica</t>
+          <t>Comunicación</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Memoria mala</t>
+          <t>Desconfiguracion</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>Electrónica</t>
+          <t>Comunicación</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Válvulas sin Voltaje</t>
+          <t>Intervencion de terceros</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>Electrónica</t>
+          <t>Comunicación</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Router sin Voltaje</t>
+          <t>Revisión tecnica</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>Electrónica</t>
+          <t>Comunicación</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Placa RS232 LAN sin voltaje</t>
+          <t>Up grade</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>Electrónica</t>
+          <t>Comunicación</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Intervencion de terceros</t>
+          <t>Cable de Red Dañado</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
-          <t>Electrónica</t>
+          <t>Construccion</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Cortocircuito</t>
+          <t>Reparación Camara</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>Electrónica</t>
+          <t>Construccion</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Revisión tecnica</t>
+          <t>Canalización</t>
         </is>
       </c>
     </row>
@@ -4574,7 +5321,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sensor de movimiento</t>
+          <t>Componente dañado</t>
         </is>
       </c>
     </row>
@@ -4586,223 +5333,223 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Up grade</t>
+          <t>Ruido</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
-          <t>Comunicación</t>
+          <t>Electrónica</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Max 232</t>
+          <t>Placa Pegada</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="inlineStr">
         <is>
-          <t>Comunicación</t>
+          <t>Electrónica</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Placa Conversor RS232 mala</t>
+          <t>Reloj Malo</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
         <is>
-          <t>Comunicación</t>
+          <t>Electrónica</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Conector DB9</t>
+          <t>Memoria mala</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>Comunicación</t>
+          <t>Electrónica</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Router</t>
+          <t>Válvulas sin Voltaje</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>Comunicación</t>
+          <t>Electrónica</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Amplimax</t>
+          <t>Router sin Voltaje</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" t="inlineStr">
         <is>
-          <t>Comunicación</t>
+          <t>Electrónica</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Placa RS232 LAN sin voltaje</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>Comunicación</t>
+          <t>Electrónica</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Conector tx rx</t>
+          <t>Intervencion de terceros</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>Comunicación</t>
+          <t>Electrónica</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ID Erróneo</t>
+          <t>Cortocircuito</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>Comunicación</t>
+          <t>Electrónica</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Desconfiguracion </t>
+          <t>Revisión tecnica</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
-          <t>Comunicación</t>
+          <t>Electrónica</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Intervencion de terceros</t>
+          <t>Sensor de movimiento</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
-          <t>Comunicación</t>
+          <t>Electrónica</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Revisión tecnica</t>
+          <t>Up grade</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" t="inlineStr">
         <is>
-          <t>Comunicación</t>
+          <t>Eléctrica</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Up grade</t>
+          <t>Cortocircuito</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" t="inlineStr">
         <is>
-          <t>Comunicación</t>
+          <t>Eléctrica</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Cable de Red Dañado</t>
+          <t>Empalme electrico</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" t="inlineStr">
         <is>
-          <t>Hídrica</t>
+          <t>Eléctrica</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Sensor de Pulso</t>
+          <t>Fusible Cortado</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" t="inlineStr">
         <is>
-          <t>Hídrica</t>
+          <t>Eléctrica</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Medidor defectuoso</t>
+          <t>Falla Fuente switching</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" t="inlineStr">
         <is>
-          <t>Hídrica</t>
+          <t>Eléctrica</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>By Pass abierto</t>
+          <t>Intervencion de terceros</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" t="inlineStr">
         <is>
-          <t>Hídrica</t>
+          <t>Eléctrica</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Solenoide</t>
+          <t>Cargador Solar</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" t="inlineStr">
         <is>
-          <t>Hídrica</t>
+          <t>Eléctrica</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Membrana</t>
+          <t>Bateria Descargada</t>
         </is>
       </c>
     </row>
@@ -4814,7 +5561,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Regulación</t>
+          <t>Sensor de Pulso</t>
         </is>
       </c>
     </row>
@@ -4826,7 +5573,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Reparación</t>
+          <t>Medidor defectuoso</t>
         </is>
       </c>
     </row>
@@ -4838,7 +5585,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Intervencion de terceros</t>
+          <t>By Pass abierto</t>
         </is>
       </c>
     </row>
@@ -4850,7 +5597,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Revisión tecnica</t>
+          <t>Solenoide</t>
         </is>
       </c>
     </row>
@@ -4862,7 +5609,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Llave de paso</t>
+          <t>Membrana</t>
         </is>
       </c>
     </row>
@@ -4874,7 +5621,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Valvula</t>
+          <t>Regulación</t>
         </is>
       </c>
     </row>
@@ -4886,7 +5633,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Fatiga de material</t>
+          <t>Reparación</t>
         </is>
       </c>
     </row>
@@ -4898,115 +5645,115 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Habilitacion CPA</t>
+          <t>Intervencion de terceros</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Hídrica</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Pick Dañado</t>
+          <t>Revisión tecnica</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Hídrica</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Actualizacion de Código</t>
+          <t>Llave de paso</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Hídrica</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Desprogramacion</t>
+          <t>Valvula</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Hídrica</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Descalibracion Peso Pulso</t>
+          <t>Fatiga de material</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" t="inlineStr">
         <is>
-          <t>Auditoría</t>
+          <t>Hídrica</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Toma de Lectura Inicial</t>
+          <t>Habilitacion CPA</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" t="inlineStr">
         <is>
-          <t>Auditoría</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Toma de Lectura Final</t>
+          <t>Pick Dañado</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" t="inlineStr">
         <is>
-          <t>Auditoría</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Validación Data</t>
+          <t>Actualizacion de Código</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
-          <t>Ultrasonido</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Renovación Silicona</t>
+          <t>Desprogramacion</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" t="inlineStr">
         <is>
-          <t>Ultrasonido</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Transductor Defectuoso</t>
+          <t>Descalibracion Peso Pulso</t>
         </is>
       </c>
     </row>
@@ -5018,7 +5765,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Q bajo 60%</t>
+          <t>Renovación Silicona</t>
         </is>
       </c>
     </row>
@@ -5030,7 +5777,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Desconfiguracion</t>
+          <t>Transductor Defectuoso</t>
         </is>
       </c>
     </row>
@@ -5042,7 +5789,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Equipo Dañado</t>
+          <t>Q bajo 60%</t>
         </is>
       </c>
     </row>
@@ -5054,71 +5801,43 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Instalación</t>
+          <t>Desconfiguracion</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Up grade </t>
+          <t>Ultrasonido</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Instalación</t>
+          <t>Equipo Dañado</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Construccion </t>
+          <t>Ultrasonido</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Reparación Camara</t>
+          <t>Instalación</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Construccion </t>
+          <t>Up grade</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Canalización</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Tareas Miscelaneas</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Retiro Sistema CIR</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Retiro Sistema CPA</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Retiro poste Solar</t>
+          <t>Instalación</t>
         </is>
       </c>
     </row>
@@ -5127,7 +5846,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5142,7 +5861,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="20">
-        <f>IFERROR(FILTER(Base3!B2:C67,Base3!B2:B67=Ingreso!C14),"")</f>
+        <f>IFERROR(FILTER(Base3!B2:C63,Base3!B2:B63=Ingreso!C14),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync visit form catalogs, drop EYES, add folio from 2250.
Refresh client/machine lists from the master sheet, remove EYES from
installed technologies, and assign correlative Folio starting at 2250
in the web form and Excel/Sheet rows.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mantenimiento_wes/FORMULARIO_MANTENCION_WES_DIGITAL.xlsx
+++ b/mantenimiento_wes/FORMULARIO_MANTENCION_WES_DIGITAL.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ingreso" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formulario Visita" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base1" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base2" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base3" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base 4" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ingreso" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Datos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Resumen" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Formulario Visita" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Base1" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Base2" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Base3" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Base 4" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Datos'!$B$1:$U$2000</definedName>
@@ -777,7 +777,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Catálogos sincronizados: 2026-08-12 19:45 desde analisis_falla_google.xlsx · 28 clientes · 159 máquinas · 62 fallas</t>
+          <t>Catálogos sincronizados: 2026-08-13 16:16 desde analisis_falla_google.xlsx · 29 clientes · 165 máquinas · 62 fallas</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C160"/>
+  <dimension ref="B1:C166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -3246,48 +3246,48 @@
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>BUPA ANTOFGASTA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CALLE DE SERVICO</t>
+          <t>MEDIDOR PRINCIPAL SANITARIA</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>BUPA ANTOFGASTA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CLUB HOUSE</t>
+          <t>SALA DE BOMBA N°2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>BUPA ANTOFGASTA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>EDIFICIO DEPORTIVO</t>
+          <t>SALA DE BOMBA SEXTO PISO</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>BUPA ANTOFGASTA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>EDIFIO DEPORTIVO</t>
+          <t>SALA DE BOMBAS PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -3299,7 +3299,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>EQUITACION</t>
+          <t>CALLE DE SERVICO</t>
         </is>
       </c>
     </row>
@@ -3311,55 +3311,55 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>RAIMUNDO TUPPER</t>
+          <t>CLUB HOUSE</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>COSTANERA</t>
+          <t>EDIFICIO DEPORTIVO</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ESTANQUE DE REUTILIZACION</t>
+          <t>EDIFIO DEPORTIVO</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LAVADO AUTO SERVICIO NORTE</t>
+          <t>EQUITACION</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>LAVADO AUTO SERVICIO SUR</t>
+          <t>RAIMUNDO TUPPER</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>LAVADO AUTOMATICO NORTE</t>
+          <t>COSTANERA</t>
         </is>
       </c>
     </row>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>LAVADO AUTOMATICO SUR</t>
+          <t>ESTANQUE DE REUTILIZACION</t>
         </is>
       </c>
     </row>
@@ -3395,7 +3395,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>LAVADO AUTO SERVICIO NORTE</t>
         </is>
       </c>
     </row>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>OFICINA ADMIN</t>
+          <t>LAVADO AUTO SERVICIO SUR</t>
         </is>
       </c>
     </row>
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PRONTO BAÑO</t>
+          <t>LAVADO AUTOMATICO NORTE</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3431,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PRONTO TIENDA</t>
+          <t>LAVADO AUTOMATICO SUR</t>
         </is>
       </c>
     </row>
@@ -3443,55 +3443,55 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>RIEGO</t>
+          <t>MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>COMPLEJO EDUCACIONAL CONSOLIDADA</t>
+          <t>OFICINA ADMIN</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ESCUELA ANDES DEL SUR</t>
+          <t>PRONTO BAÑO</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ESCUELA GABRIELA</t>
+          <t>PRONTO TIENDA</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ESCUELA JUAN MACKENNA</t>
+          <t>RIEGO</t>
         </is>
       </c>
     </row>
@@ -3503,7 +3503,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ESCUELA LOS ANDES</t>
+          <t>COMPLEJO EDUCACIONAL CONSOLIDADA</t>
         </is>
       </c>
     </row>
@@ -3515,7 +3515,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ESCUELA LUIS MATTE LARRAIN</t>
+          <t>ESCUELA ANDES DEL SUR</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3527,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ESCUELA PADRE HURTADO</t>
+          <t>ESCUELA GABRIELA</t>
         </is>
       </c>
     </row>
@@ -3539,7 +3539,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ESCUELA VILLA INDEPENDENCIA</t>
+          <t>ESCUELA JUAN MACKENNA</t>
         </is>
       </c>
     </row>
@@ -3551,7 +3551,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ESCULA NONATO COO</t>
+          <t>ESCUELA LOS ANDES</t>
         </is>
       </c>
     </row>
@@ -3563,7 +3563,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LICEO CHILOE</t>
+          <t>ESCUELA LUIS MATTE LARRAIN</t>
         </is>
       </c>
     </row>
@@ -3575,55 +3575,55 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>LICEO MAIPO</t>
+          <t>ESCUELA PADRE HURTADO</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ALICURA</t>
+          <t>ESCUELA VILLA INDEPENDENCIA</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ANTONIO HERMIDA FABRES</t>
+          <t>ESCULA NONATO COO</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CARLOS FERNANDEZ PEÑA</t>
+          <t>LICEO CHILOE</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CENTRO EDUCACIONAL EDUARDO DE LA BARRA</t>
+          <t>LICEO MAIPO</t>
         </is>
       </c>
     </row>
@@ -3635,7 +3635,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>CENTRO EDUCACIONAL VALLE HERMOSO</t>
+          <t>ALICURA</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ERASMO ESCALA</t>
+          <t>ANTONIO HERMIDA FABRES</t>
         </is>
       </c>
     </row>
@@ -3659,7 +3659,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ESCUELA ESPECIAL PONTÍFICE JUAN PABLO II</t>
+          <t>CARLOS FERNANDEZ PEÑA</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ESCUELA LUIS ARRIETA CAÑAS</t>
+          <t>CENTRO EDUCACIONAL EDUARDO DE LA BARRA</t>
         </is>
       </c>
     </row>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ESCUELA UNIÓN NACIONAL ÁRABE</t>
+          <t>CENTRO EDUCACIONAL VALLE HERMOSO</t>
         </is>
       </c>
     </row>
@@ -3695,7 +3695,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>JUAN BAUTISTA PASTENE</t>
+          <t>ERASMO ESCALA</t>
         </is>
       </c>
     </row>
@@ -3707,7 +3707,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>LIKANKURA</t>
+          <t>ESCUELA ESPECIAL PONTÍFICE JUAN PABLO II</t>
         </is>
       </c>
     </row>
@@ -3719,7 +3719,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>MATILDE HUICI NAVAS</t>
+          <t>ESCUELA LUIS ARRIETA CAÑAS</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3731,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>SANTA MARIA</t>
+          <t>ESCUELA UNIÓN NACIONAL ÁRABE</t>
         </is>
       </c>
     </row>
@@ -3743,79 +3743,79 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>TOBALABA</t>
+          <t>JUAN BAUTISTA PASTENE</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" t="inlineStr">
         <is>
-          <t>CUR</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ANILLO NORTE</t>
+          <t>LIKANKURA</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" t="inlineStr">
         <is>
-          <t>CUR</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ANILLO SUR</t>
+          <t>MATILDE HUICI NAVAS</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
-          <t>CUR</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>BAÑOS</t>
+          <t>SANTA MARIA</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" t="inlineStr">
         <is>
-          <t>CUR</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>TOBALABA</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>CUR</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>LO BOZA - EDIFICIO PRINCIPAL CASINO</t>
+          <t>ANILLO NORTE</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="B58" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>CUR</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>LO BOZA - LAVADO DE VEHICULOS</t>
+          <t>ANILLO SUR</t>
         </is>
       </c>
     </row>
@@ -3827,7 +3827,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>LO BOZA - POZO DE LAVADO DE VEHICULO</t>
+          <t>LO BOZA - EDIFICIO PRINCIPAL CASINO</t>
         </is>
       </c>
     </row>
@@ -3839,7 +3839,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>LO BOZA - REUTILIZACION</t>
+          <t>LO BOZA - LAVADO DE VEHICULOS</t>
         </is>
       </c>
     </row>
@@ -3851,7 +3851,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>LO BOZA - SALA DE IMPULSION</t>
+          <t>LO BOZA - POZO DE LAVADO DE VEHICULO</t>
         </is>
       </c>
     </row>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>OPEN PLAZA - MATRIZ PRINCIPAL</t>
+          <t>LO BOZA - REUTILIZACION</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>PRONTO BAÑO</t>
+          <t>LO BOZA - SALA DE IMPULSION</t>
         </is>
       </c>
     </row>
@@ -3887,7 +3887,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>QUILICURA - CAMARINES</t>
+          <t>OPEN PLAZA - MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -3899,7 +3899,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>QUILICURA - CASINO</t>
+          <t>PRONTO BAÑO</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>QUILICURA - DERCOMAQ</t>
+          <t>QUILICURA - CAMARINES</t>
         </is>
       </c>
     </row>
@@ -3923,7 +3923,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>QUILICURA - EDIFICIO JCB</t>
+          <t>QUILICURA - CASINO</t>
         </is>
       </c>
     </row>
@@ -3935,7 +3935,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>QUILICURA - LAVADO DE MAQUINA</t>
+          <t>QUILICURA - DERCOMAQ</t>
         </is>
       </c>
     </row>
@@ -3947,7 +3947,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>QUILICURA - MATRIZ PRINCIPAL</t>
+          <t>QUILICURA - EDIFICIO JCB</t>
         </is>
       </c>
     </row>
@@ -3959,55 +3959,55 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>QUILICURA - PRODERCO</t>
+          <t>QUILICURA - LAVADO DE MAQUINA</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="B71" t="inlineStr">
         <is>
-          <t>ESTADIO ISRAELITA</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>MATRIS CHESTERTON</t>
+          <t>QUILICURA - MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="B72" t="inlineStr">
         <is>
-          <t>ESTADIO ISRAELITA</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>MATRIZ AV LAS CONDES</t>
+          <t>QUILICURA - PRODERCO</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="B73" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>ESTADIO ISRAELITA</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>ETAPA 1,2,3 Y 4</t>
+          <t>MATRIS CHESTERTON</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="B74" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>ESTADIO ISRAELITA</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ETAPA 5</t>
+          <t>MATRIZ AV LAS CONDES</t>
         </is>
       </c>
     </row>
@@ -4019,7 +4019,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>MATRIS ESVAL</t>
+          <t>ESTANQUE INFERIOR</t>
         </is>
       </c>
     </row>
@@ -4031,91 +4031,91 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>RIEGO</t>
+          <t>ETAPA 1</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="B77" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>CDP PUENTE ALTO</t>
+          <t>ETAPA 1,2,3 Y 4</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="B78" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>COLINA 1</t>
+          <t>ETAPA 1-4</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="B79" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>COLINA 2 RED SUR</t>
+          <t>ETAPA 2</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="B80" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>COLINA 2 REDIMPULSION</t>
+          <t>ETAPA 3</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="B81" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>CPA MODULO</t>
+          <t>ETAPA 5</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="B82" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>CPA OVALO</t>
+          <t>MATRIS ESVAL</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="B83" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>CPF SAN MIGUEL MATRIZ PRINCIPAL</t>
+          <t>RIEGO LLENADO DE ESTANQUE ESVAL</t>
         </is>
       </c>
     </row>
@@ -4127,7 +4127,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>CPF SAN MIGUEL SALA IMPULSION</t>
+          <t>CDP PUENTE ALTO</t>
         </is>
       </c>
     </row>
@@ -4139,7 +4139,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ESC. EL BOSQUE ADMINISTRACION</t>
+          <t>COLINA 1</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>ESC. EL BOSQUE GENCHI ACADEMIA</t>
+          <t>COLINA 2 RED SUR</t>
         </is>
       </c>
     </row>
@@ -4163,7 +4163,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ESC. OF ARTEMIO</t>
+          <t>COLINA 2 REDIMPULSION</t>
         </is>
       </c>
     </row>
@@ -4175,7 +4175,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ESC. OF CARMEN</t>
+          <t>CPA MODULO</t>
         </is>
       </c>
     </row>
@@ -4187,7 +4187,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>ESCUELA ANDES DEL SUR</t>
+          <t>CPA OVALO</t>
         </is>
       </c>
     </row>
@@ -4199,7 +4199,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>ESFORPEN BOSQUE ADMINISTRACION</t>
+          <t>CPF SAN MIGUEL MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>ESFORPEN BOSQUE GENCHI SIMULACION</t>
+          <t>CPF SAN MIGUEL SALA IMPULSION</t>
         </is>
       </c>
     </row>
@@ -4223,7 +4223,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>MONITOREO MATRIZ PRINCIPAL MODULO</t>
+          <t>ESC. EL BOSQUE ADMINISTRACION</t>
         </is>
       </c>
     </row>
@@ -4235,499 +4235,499 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>MONITOREO MATRIZ PRINCIPAL OVALO</t>
+          <t>ESC. EL BOSQUE GENCHI ACADEMIA</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="B94" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>AGUA BLANDA</t>
+          <t>ESC. OF ARTEMIO</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="B95" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>INTERCAMBIADOR 1</t>
+          <t>ESC. OF CARMEN</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="B96" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>INTERCAMBIADOR 2</t>
+          <t>ESCUELA ANDES DEL SUR</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="B97" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>ESFORPEN BOSQUE ADMINISTRACION</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="B98" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>RETORNO OSMOSIS</t>
+          <t>ESFORPEN BOSQUE GENCHI SIMULACION</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="B99" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>SALIDA OSMOSIS</t>
+          <t>MONITOREO MATRIZ PRINCIPAL MODULO</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="B100" t="inlineStr">
         <is>
-          <t>LA FLORIDA</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>LICEO ALTO CORDILLERA</t>
+          <t>MONITOREO MATRIZ PRINCIPAL OVALO</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="B101" t="inlineStr">
         <is>
-          <t>LA REINA</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>EUGENIO MARIA DE HOSTOS</t>
+          <t>AGUA BLANDA</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>LAS CONDES</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>FLEMING</t>
+          <t>INTERCAMBIADOR 1</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="B103" t="inlineStr">
         <is>
-          <t>LAS CONDES</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>JUAN PABLO II</t>
+          <t>INTERCAMBIADOR 2</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
-          <t>LAS CONDES</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>LIKANKURA</t>
+          <t>MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="B105" t="inlineStr">
         <is>
-          <t>LO VALLEDOR</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>BARRIO NORTE</t>
+          <t>RETORNO OSMOSIS</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="B106" t="inlineStr">
         <is>
-          <t>LO VALLEDOR</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>POZO 1</t>
+          <t>SALIDA OSMOSIS</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="B107" t="inlineStr">
         <is>
-          <t>LO VALLEDOR</t>
+          <t>LA FLORIDA</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>PUERTA 1</t>
+          <t>LICEO ALTO CORDILLERA</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="B108" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>LA REINA</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>CASINO</t>
+          <t>EUGENIO MARIA DE HOSTOS</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>LAS CONDES</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>ESTANQUE CISTERNA</t>
+          <t>FLEMING</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="B110" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>LAS CONDES</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>SAN NICOLAS</t>
+          <t>JUAN PABLO II</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="B111" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>LAS CONDES</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>URETA COX</t>
+          <t>LIKANKURA</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="B112" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>LO VALLEDOR</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>BAÑO GUARDIAS</t>
+          <t>BARRIO NORTE</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="B113" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>LO VALLEDOR</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
+          <t>POZO 1</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="B114" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>LO VALLEDOR</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>ESTANQUE NORTE LOCALES</t>
+          <t>PUERTA 1</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="B115" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>ESTANQUE SUR ABASTECIMIENTO</t>
+          <t>CASINO</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="B116" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>KFC</t>
+          <t>ESTANQUE CISTERNA</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="B117" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>PIZZA HUT</t>
+          <t>SAN NICOLAS</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="B118" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>MATRIZ BOULEVARD PASILLO TECNICO</t>
+          <t>URETA COX</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="B119" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>MATRIZ SALIDA DE EMERGENCIA PASILLO N°1 ARROW</t>
+          <t>BAÑO GUARDIAS</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="B120" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>PLACA BANCARIA</t>
+          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="B121" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS FALABELLA</t>
+          <t>ESTANQUE NORTE LOCALES</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="B122" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS RIPLEY</t>
+          <t>KFC</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="B123" t="inlineStr">
         <is>
-          <t>MAQ</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>ALIMENTACION DE BAÑOS</t>
+          <t>PIZZA HUT</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="B124" t="inlineStr">
         <is>
-          <t>MAQ</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>SALA DE BOMBAS ESTANQUE SUR</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="B125" t="inlineStr">
         <is>
-          <t>MAQ</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>RED DE INCENDIO</t>
+          <t>MATRIZ BOULEVARD PASILLO TECNICO</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="B126" t="inlineStr">
         <is>
-          <t>MOLYMET</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>CASA DE CAMBIO</t>
+          <t>MATRIZ SALIDA DE EMERGENCIA PASILLO N°1 ARROW</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="B127" t="inlineStr">
         <is>
-          <t>MOLYMET</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>RIEGO</t>
+          <t>PLACA BANCARIA</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="B128" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>CANCHA</t>
+          <t>SALA DE BOMBAS FALABELLA</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="B129" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>CONTROL NIDO</t>
+          <t>SALA DE BOMBAS RIPLEY</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="B130" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>MAQ</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ELEMENTARY</t>
+          <t>ALIMENTACION DE BAÑOS</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="B131" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>MAQ</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ESTANQUE B</t>
+          <t>MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="B132" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>MAQ</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>ESTANQUE C</t>
+          <t>RED DE INCENDIO</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="B133" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>MOLYMET</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>HIGH SCHOOL</t>
+          <t>CASA DE CAMBIO</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="B134" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>MOLYMET</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>PISCINA</t>
+          <t>RIEGO</t>
         </is>
       </c>
     </row>
@@ -4739,7 +4739,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>POZO PROFUNDO</t>
+          <t>CANCHA</t>
         </is>
       </c>
     </row>
@@ -4751,139 +4751,139 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>TEATRO</t>
+          <t>CONTROL NIDO</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="B137" t="inlineStr">
         <is>
-          <t>PAE</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
+          <t>ELEMENTARY</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="B138" t="inlineStr">
         <is>
-          <t>PAE</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>ESTANQUE NORTE LOCALES</t>
+          <t>ESTANQUE B</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="B139" t="inlineStr">
         <is>
-          <t>PAE</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>KFC</t>
+          <t>ESTANQUE C</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="B140" t="inlineStr">
         <is>
-          <t>PAE</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>PIZZA HUT</t>
+          <t>HIGH SCHOOL</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="B141" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>ANDEN 3-4 LOCALES GASTRONOMICOS</t>
+          <t>PISCINA</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="B142" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>ANDEN 3-4 MATRIZ PRINCIPAL</t>
+          <t>POZO PROFUNDO</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="B143" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>ANDEN 3-4 RESTAURANTE</t>
+          <t>TEATRO</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="B144" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>BAZAR GOURMET</t>
+          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="B145" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>BAÑO DAMAS</t>
+          <t>ESTANQUE NORTE LOCALES</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="B146" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>BAÑO VARONES</t>
+          <t>KFC</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="B147" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>DISTRITO DE LUJO</t>
+          <t>PIZZA HUT</t>
         </is>
       </c>
     </row>
@@ -4895,7 +4895,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>DL KENNEDY</t>
+          <t>ANDEN 3-4 LOCALES GASTRONOMICOS</t>
         </is>
       </c>
     </row>
@@ -4907,7 +4907,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>LLENADO DE PILETA</t>
+          <t>ANDEN 3-4 MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>PILETA CASCADA</t>
+          <t>ANDEN 3-4 RESTAURANTE</t>
         </is>
       </c>
     </row>
@@ -4931,7 +4931,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>SANDIA ANTIGUA</t>
+          <t>BAZAR GOURMET</t>
         </is>
       </c>
     </row>
@@ -4943,101 +4943,173 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>SANDIA NUEVA</t>
+          <t>DISTRITO DE LUJO</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="B153" t="inlineStr">
         <is>
-          <t>PROVIDENCIA</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>ARTURO ALESSANDRI PALMA</t>
+          <t>DL KENNEDY</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="B154" t="inlineStr">
         <is>
-          <t>PROVIDENCIA</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>CARMELA CARVAJAL</t>
+          <t>LLENADO DE PILETA</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="B155" t="inlineStr">
         <is>
-          <t>PROVIDENCIA</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>LASTARRIA</t>
+          <t>PILETA CASCADA</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="B156" t="inlineStr">
         <is>
-          <t>RENCA</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>CAPITAN JOSÉ LUIS ARANDE</t>
+          <t>SANDIA ANTIGUA</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="B157" t="inlineStr">
         <is>
-          <t>RENCA</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>JUAN DE ATALA HIRMAS</t>
+          <t>SANDIA NUEVA</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="B158" t="inlineStr">
         <is>
-          <t>RENCA</t>
+          <t>PROVIDENCIA</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>REBECA MATTE BELLO</t>
+          <t>CARMELA CARVAJAL</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="B159" t="inlineStr">
         <is>
-          <t>UDD</t>
+          <t>PROVIDENCIA</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS EDIFICIO ¨O¨</t>
+          <t>LASTARRIA</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="B160" t="inlineStr">
         <is>
+          <t>PROVIDENCIA</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>LICEO JUAN PABLO DUARTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>PROVIDENCIA</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>LICEO N°7</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>CAPITAN JOSÉ LUIS ARANDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>JUAN DE ATALA HIRMAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>REBECA MATTE BELLO</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="B165" t="inlineStr">
+        <is>
           <t>UDD</t>
         </is>
       </c>
-      <c r="C160" t="inlineStr">
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>SALA DE BOMBAS EDIFICIO ¨O¨</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>UDD</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
         <is>
           <t>SALA DE BOMBAS HONDURAS</t>
         </is>
@@ -5063,7 +5135,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="20">
-        <f>IFERROR(FILTER(Base1!B2:C160,Base1!B2:B160=Ingreso!C4),"")</f>
+        <f>IFERROR(FILTER(Base1!B2:C166,Base1!B2:B166=Ingreso!C4),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync catalogs: add CDUC CANCHAS DE TENIS to visit form.
Redeployed Apps Script web app so technicians see the new machine in the dropdown.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mantenimiento_wes/FORMULARIO_MANTENCION_WES_DIGITAL.xlsx
+++ b/mantenimiento_wes/FORMULARIO_MANTENCION_WES_DIGITAL.xlsx
@@ -777,7 +777,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Catálogos sincronizados: 2026-08-13 16:16 desde analisis_falla_google.xlsx · 29 clientes · 165 máquinas · 62 fallas</t>
+          <t>Catálogos sincronizados: 2026-08-13 17:49 desde analisis_falla_google.xlsx · 29 clientes · 166 máquinas · 62 fallas</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C166"/>
+  <dimension ref="B1:C167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -3311,7 +3311,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CLUB HOUSE</t>
+          <t>CANCHAS DE TENIS</t>
         </is>
       </c>
     </row>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>EDIFICIO DEPORTIVO</t>
+          <t>CLUB HOUSE</t>
         </is>
       </c>
     </row>
@@ -3335,7 +3335,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>EDIFIO DEPORTIVO</t>
+          <t>EDIFICIO DEPORTIVO</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>EQUITACION</t>
+          <t>EDIFIO DEPORTIVO</t>
         </is>
       </c>
     </row>
@@ -3359,19 +3359,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>RAIMUNDO TUPPER</t>
+          <t>EQUITACION</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>COSTANERA</t>
+          <t>RAIMUNDO TUPPER</t>
         </is>
       </c>
     </row>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ESTANQUE DE REUTILIZACION</t>
+          <t>COSTANERA</t>
         </is>
       </c>
     </row>
@@ -3395,7 +3395,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>LAVADO AUTO SERVICIO NORTE</t>
+          <t>ESTANQUE DE REUTILIZACION</t>
         </is>
       </c>
     </row>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>LAVADO AUTO SERVICIO SUR</t>
+          <t>LAVADO AUTO SERVICIO NORTE</t>
         </is>
       </c>
     </row>
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LAVADO AUTOMATICO NORTE</t>
+          <t>LAVADO AUTO SERVICIO SUR</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3431,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LAVADO AUTOMATICO SUR</t>
+          <t>LAVADO AUTOMATICO NORTE</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>LAVADO AUTOMATICO SUR</t>
         </is>
       </c>
     </row>
@@ -3455,7 +3455,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>OFICINA ADMIN</t>
+          <t>MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -3467,7 +3467,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PRONTO BAÑO</t>
+          <t>OFICINA ADMIN</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PRONTO TIENDA</t>
+          <t>PRONTO BAÑO</t>
         </is>
       </c>
     </row>
@@ -3491,19 +3491,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>RIEGO</t>
+          <t>PRONTO TIENDA</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>COMPLEJO EDUCACIONAL CONSOLIDADA</t>
+          <t>RIEGO</t>
         </is>
       </c>
     </row>
@@ -3515,7 +3515,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ESCUELA ANDES DEL SUR</t>
+          <t>COMPLEJO EDUCACIONAL CONSOLIDADA</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3527,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ESCUELA GABRIELA</t>
+          <t>ESCUELA ANDES DEL SUR</t>
         </is>
       </c>
     </row>
@@ -3539,7 +3539,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ESCUELA JUAN MACKENNA</t>
+          <t>ESCUELA GABRIELA</t>
         </is>
       </c>
     </row>
@@ -3551,7 +3551,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ESCUELA LOS ANDES</t>
+          <t>ESCUELA JUAN MACKENNA</t>
         </is>
       </c>
     </row>
@@ -3563,7 +3563,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ESCUELA LUIS MATTE LARRAIN</t>
+          <t>ESCUELA LOS ANDES</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ESCUELA PADRE HURTADO</t>
+          <t>ESCUELA LUIS MATTE LARRAIN</t>
         </is>
       </c>
     </row>
@@ -3587,7 +3587,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ESCUELA VILLA INDEPENDENCIA</t>
+          <t>ESCUELA PADRE HURTADO</t>
         </is>
       </c>
     </row>
@@ -3599,7 +3599,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ESCULA NONATO COO</t>
+          <t>ESCUELA VILLA INDEPENDENCIA</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>LICEO CHILOE</t>
+          <t>ESCULA NONATO COO</t>
         </is>
       </c>
     </row>
@@ -3623,19 +3623,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LICEO MAIPO</t>
+          <t>LICEO CHILOE</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ALICURA</t>
+          <t>LICEO MAIPO</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ANTONIO HERMIDA FABRES</t>
+          <t>ALICURA</t>
         </is>
       </c>
     </row>
@@ -3659,7 +3659,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>CARLOS FERNANDEZ PEÑA</t>
+          <t>ANTONIO HERMIDA FABRES</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>CENTRO EDUCACIONAL EDUARDO DE LA BARRA</t>
+          <t>CARLOS FERNANDEZ PEÑA</t>
         </is>
       </c>
     </row>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CENTRO EDUCACIONAL VALLE HERMOSO</t>
+          <t>CENTRO EDUCACIONAL EDUARDO DE LA BARRA</t>
         </is>
       </c>
     </row>
@@ -3695,7 +3695,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ERASMO ESCALA</t>
+          <t>CENTRO EDUCACIONAL VALLE HERMOSO</t>
         </is>
       </c>
     </row>
@@ -3707,7 +3707,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ESCUELA ESPECIAL PONTÍFICE JUAN PABLO II</t>
+          <t>ERASMO ESCALA</t>
         </is>
       </c>
     </row>
@@ -3719,7 +3719,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ESCUELA LUIS ARRIETA CAÑAS</t>
+          <t>ESCUELA ESPECIAL PONTÍFICE JUAN PABLO II</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3731,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ESCUELA UNIÓN NACIONAL ÁRABE</t>
+          <t>ESCUELA LUIS ARRIETA CAÑAS</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>JUAN BAUTISTA PASTENE</t>
+          <t>ESCUELA UNIÓN NACIONAL ÁRABE</t>
         </is>
       </c>
     </row>
@@ -3755,7 +3755,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>LIKANKURA</t>
+          <t>JUAN BAUTISTA PASTENE</t>
         </is>
       </c>
     </row>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>MATILDE HUICI NAVAS</t>
+          <t>LIKANKURA</t>
         </is>
       </c>
     </row>
@@ -3779,7 +3779,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>SANTA MARIA</t>
+          <t>MATILDE HUICI NAVAS</t>
         </is>
       </c>
     </row>
@@ -3791,19 +3791,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>TOBALABA</t>
+          <t>SANTA MARIA</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" t="inlineStr">
         <is>
-          <t>CUR</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ANILLO NORTE</t>
+          <t>TOBALABA</t>
         </is>
       </c>
     </row>
@@ -3815,19 +3815,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ANILLO SUR</t>
+          <t>ANILLO NORTE</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>CUR</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>LO BOZA - EDIFICIO PRINCIPAL CASINO</t>
+          <t>ANILLO SUR</t>
         </is>
       </c>
     </row>
@@ -3839,7 +3839,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>LO BOZA - LAVADO DE VEHICULOS</t>
+          <t>LO BOZA - EDIFICIO PRINCIPAL CASINO</t>
         </is>
       </c>
     </row>
@@ -3851,7 +3851,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>LO BOZA - POZO DE LAVADO DE VEHICULO</t>
+          <t>LO BOZA - LAVADO DE VEHICULOS</t>
         </is>
       </c>
     </row>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>LO BOZA - REUTILIZACION</t>
+          <t>LO BOZA - POZO DE LAVADO DE VEHICULO</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>LO BOZA - SALA DE IMPULSION</t>
+          <t>LO BOZA - REUTILIZACION</t>
         </is>
       </c>
     </row>
@@ -3887,7 +3887,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>OPEN PLAZA - MATRIZ PRINCIPAL</t>
+          <t>LO BOZA - SALA DE IMPULSION</t>
         </is>
       </c>
     </row>
@@ -3899,7 +3899,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>PRONTO BAÑO</t>
+          <t>OPEN PLAZA - MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>QUILICURA - CAMARINES</t>
+          <t>PRONTO BAÑO</t>
         </is>
       </c>
     </row>
@@ -3923,7 +3923,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>QUILICURA - CASINO</t>
+          <t>QUILICURA - CAMARINES</t>
         </is>
       </c>
     </row>
@@ -3935,7 +3935,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>QUILICURA - DERCOMAQ</t>
+          <t>QUILICURA - CASINO</t>
         </is>
       </c>
     </row>
@@ -3947,7 +3947,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>QUILICURA - EDIFICIO JCB</t>
+          <t>QUILICURA - DERCOMAQ</t>
         </is>
       </c>
     </row>
@@ -3959,7 +3959,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>QUILICURA - LAVADO DE MAQUINA</t>
+          <t>QUILICURA - EDIFICIO JCB</t>
         </is>
       </c>
     </row>
@@ -3971,7 +3971,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>QUILICURA - MATRIZ PRINCIPAL</t>
+          <t>QUILICURA - LAVADO DE MAQUINA</t>
         </is>
       </c>
     </row>
@@ -3983,19 +3983,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>QUILICURA - PRODERCO</t>
+          <t>QUILICURA - MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="B73" t="inlineStr">
         <is>
-          <t>ESTADIO ISRAELITA</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>MATRIS CHESTERTON</t>
+          <t>QUILICURA - PRODERCO</t>
         </is>
       </c>
     </row>
@@ -4007,19 +4007,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>MATRIZ AV LAS CONDES</t>
+          <t>MATRIS CHESTERTON</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="B75" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>ESTADIO ISRAELITA</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ESTANQUE INFERIOR</t>
+          <t>MATRIZ AV LAS CONDES</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ETAPA 1</t>
+          <t>ESTANQUE INFERIOR</t>
         </is>
       </c>
     </row>
@@ -4043,7 +4043,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ETAPA 1,2,3 Y 4</t>
+          <t>ETAPA 1</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4055,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ETAPA 1-4</t>
+          <t>ETAPA 1,2,3 Y 4</t>
         </is>
       </c>
     </row>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>ETAPA 2</t>
+          <t>ETAPA 1-4</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4079,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>ETAPA 3</t>
+          <t>ETAPA 2</t>
         </is>
       </c>
     </row>
@@ -4091,7 +4091,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ETAPA 5</t>
+          <t>ETAPA 3</t>
         </is>
       </c>
     </row>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>MATRIS ESVAL</t>
+          <t>ETAPA 5</t>
         </is>
       </c>
     </row>
@@ -4115,19 +4115,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>RIEGO LLENADO DE ESTANQUE ESVAL</t>
+          <t>MATRIS ESVAL</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="B84" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>CDP PUENTE ALTO</t>
+          <t>RIEGO LLENADO DE ESTANQUE ESVAL</t>
         </is>
       </c>
     </row>
@@ -4139,7 +4139,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>COLINA 1</t>
+          <t>CDP PUENTE ALTO</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>COLINA 2 RED SUR</t>
+          <t>COLINA 1</t>
         </is>
       </c>
     </row>
@@ -4163,7 +4163,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>COLINA 2 REDIMPULSION</t>
+          <t>COLINA 2 RED SUR</t>
         </is>
       </c>
     </row>
@@ -4175,7 +4175,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>CPA MODULO</t>
+          <t>COLINA 2 REDIMPULSION</t>
         </is>
       </c>
     </row>
@@ -4187,7 +4187,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>CPA OVALO</t>
+          <t>CPA MODULO</t>
         </is>
       </c>
     </row>
@@ -4199,7 +4199,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>CPF SAN MIGUEL MATRIZ PRINCIPAL</t>
+          <t>CPA OVALO</t>
         </is>
       </c>
     </row>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>CPF SAN MIGUEL SALA IMPULSION</t>
+          <t>CPF SAN MIGUEL MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -4223,7 +4223,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>ESC. EL BOSQUE ADMINISTRACION</t>
+          <t>CPF SAN MIGUEL SALA IMPULSION</t>
         </is>
       </c>
     </row>
@@ -4235,7 +4235,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>ESC. EL BOSQUE GENCHI ACADEMIA</t>
+          <t>ESC. EL BOSQUE ADMINISTRACION</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>ESC. OF ARTEMIO</t>
+          <t>ESC. EL BOSQUE GENCHI ACADEMIA</t>
         </is>
       </c>
     </row>
@@ -4259,7 +4259,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>ESC. OF CARMEN</t>
+          <t>ESC. OF ARTEMIO</t>
         </is>
       </c>
     </row>
@@ -4271,7 +4271,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>ESCUELA ANDES DEL SUR</t>
+          <t>ESC. OF CARMEN</t>
         </is>
       </c>
     </row>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>ESFORPEN BOSQUE ADMINISTRACION</t>
+          <t>ESCUELA ANDES DEL SUR</t>
         </is>
       </c>
     </row>
@@ -4295,7 +4295,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>ESFORPEN BOSQUE GENCHI SIMULACION</t>
+          <t>ESFORPEN BOSQUE ADMINISTRACION</t>
         </is>
       </c>
     </row>
@@ -4307,7 +4307,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>MONITOREO MATRIZ PRINCIPAL MODULO</t>
+          <t>ESFORPEN BOSQUE GENCHI SIMULACION</t>
         </is>
       </c>
     </row>
@@ -4319,19 +4319,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>MONITOREO MATRIZ PRINCIPAL OVALO</t>
+          <t>MONITOREO MATRIZ PRINCIPAL MODULO</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="B101" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>AGUA BLANDA</t>
+          <t>MONITOREO MATRIZ PRINCIPAL OVALO</t>
         </is>
       </c>
     </row>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>INTERCAMBIADOR 1</t>
+          <t>AGUA BLANDA</t>
         </is>
       </c>
     </row>
@@ -4355,7 +4355,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>INTERCAMBIADOR 2</t>
+          <t>INTERCAMBIADOR 1</t>
         </is>
       </c>
     </row>
@@ -4367,7 +4367,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>INTERCAMBIADOR 2</t>
         </is>
       </c>
     </row>
@@ -4379,7 +4379,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>RETORNO OSMOSIS</t>
+          <t>MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -4391,43 +4391,43 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>SALIDA OSMOSIS</t>
+          <t>RETORNO OSMOSIS</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="B107" t="inlineStr">
         <is>
-          <t>LA FLORIDA</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>LICEO ALTO CORDILLERA</t>
+          <t>SALIDA OSMOSIS</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="B108" t="inlineStr">
         <is>
-          <t>LA REINA</t>
+          <t>LA FLORIDA</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>EUGENIO MARIA DE HOSTOS</t>
+          <t>LICEO ALTO CORDILLERA</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
-          <t>LAS CONDES</t>
+          <t>LA REINA</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>FLEMING</t>
+          <t>EUGENIO MARIA DE HOSTOS</t>
         </is>
       </c>
     </row>
@@ -4439,7 +4439,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>JUAN PABLO II</t>
+          <t>FLEMING</t>
         </is>
       </c>
     </row>
@@ -4451,19 +4451,19 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>LIKANKURA</t>
+          <t>JUAN PABLO II</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="B112" t="inlineStr">
         <is>
-          <t>LO VALLEDOR</t>
+          <t>LAS CONDES</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>BARRIO NORTE</t>
+          <t>LIKANKURA</t>
         </is>
       </c>
     </row>
@@ -4475,7 +4475,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>POZO 1</t>
+          <t>BARRIO NORTE</t>
         </is>
       </c>
     </row>
@@ -4487,19 +4487,19 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>PUERTA 1</t>
+          <t>POZO 1</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="B115" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>LO VALLEDOR</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>CASINO</t>
+          <t>PUERTA 1</t>
         </is>
       </c>
     </row>
@@ -4511,7 +4511,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ESTANQUE CISTERNA</t>
+          <t>CASINO</t>
         </is>
       </c>
     </row>
@@ -4523,7 +4523,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>SAN NICOLAS</t>
+          <t>ESTANQUE CISTERNA</t>
         </is>
       </c>
     </row>
@@ -4535,19 +4535,19 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>URETA COX</t>
+          <t>SAN NICOLAS</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="B119" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>BAÑO GUARDIAS</t>
+          <t>URETA COX</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
+          <t>BAÑO GUARDIAS</t>
         </is>
       </c>
     </row>
@@ -4571,7 +4571,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ESTANQUE NORTE LOCALES</t>
+          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
         </is>
       </c>
     </row>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>KFC</t>
+          <t>ESTANQUE NORTE LOCALES</t>
         </is>
       </c>
     </row>
@@ -4595,7 +4595,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>PIZZA HUT</t>
+          <t>KFC</t>
         </is>
       </c>
     </row>
@@ -4607,19 +4607,19 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS ESTANQUE SUR</t>
+          <t>PIZZA HUT</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="B125" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>MATRIZ BOULEVARD PASILLO TECNICO</t>
+          <t>SALA DE BOMBAS ESTANQUE SUR</t>
         </is>
       </c>
     </row>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>MATRIZ SALIDA DE EMERGENCIA PASILLO N°1 ARROW</t>
+          <t>MATRIZ BOULEVARD PASILLO TECNICO</t>
         </is>
       </c>
     </row>
@@ -4643,7 +4643,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>PLACA BANCARIA</t>
+          <t>MATRIZ SALIDA DE EMERGENCIA PASILLO N°1 ARROW</t>
         </is>
       </c>
     </row>
@@ -4655,7 +4655,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS FALABELLA</t>
+          <t>PLACA BANCARIA</t>
         </is>
       </c>
     </row>
@@ -4667,19 +4667,19 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS RIPLEY</t>
+          <t>SALA DE BOMBAS FALABELLA</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="B130" t="inlineStr">
         <is>
-          <t>MAQ</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ALIMENTACION DE BAÑOS</t>
+          <t>SALA DE BOMBAS RIPLEY</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>ALIMENTACION DE BAÑOS</t>
         </is>
       </c>
     </row>
@@ -4703,19 +4703,19 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>RED DE INCENDIO</t>
+          <t>MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="B133" t="inlineStr">
         <is>
-          <t>MOLYMET</t>
+          <t>MAQ</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>CASA DE CAMBIO</t>
+          <t>RED DE INCENDIO</t>
         </is>
       </c>
     </row>
@@ -4727,19 +4727,19 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>RIEGO</t>
+          <t>CASA DE CAMBIO</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="B135" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>MOLYMET</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>CANCHA</t>
+          <t>RIEGO</t>
         </is>
       </c>
     </row>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>CONTROL NIDO</t>
+          <t>CANCHA</t>
         </is>
       </c>
     </row>
@@ -4763,7 +4763,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>ELEMENTARY</t>
+          <t>CONTROL NIDO</t>
         </is>
       </c>
     </row>
@@ -4775,7 +4775,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>ESTANQUE B</t>
+          <t>ELEMENTARY</t>
         </is>
       </c>
     </row>
@@ -4787,7 +4787,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ESTANQUE C</t>
+          <t>ESTANQUE B</t>
         </is>
       </c>
     </row>
@@ -4799,7 +4799,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>HIGH SCHOOL</t>
+          <t>ESTANQUE C</t>
         </is>
       </c>
     </row>
@@ -4811,7 +4811,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>PISCINA</t>
+          <t>HIGH SCHOOL</t>
         </is>
       </c>
     </row>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>POZO PROFUNDO</t>
+          <t>PISCINA</t>
         </is>
       </c>
     </row>
@@ -4835,19 +4835,19 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>TEATRO</t>
+          <t>POZO PROFUNDO</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="B144" t="inlineStr">
         <is>
-          <t>PAE</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
+          <t>TEATRO</t>
         </is>
       </c>
     </row>
@@ -4859,7 +4859,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>ESTANQUE NORTE LOCALES</t>
+          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>KFC</t>
+          <t>ESTANQUE NORTE LOCALES</t>
         </is>
       </c>
     </row>
@@ -4883,19 +4883,19 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>PIZZA HUT</t>
+          <t>KFC</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="B148" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>ANDEN 3-4 LOCALES GASTRONOMICOS</t>
+          <t>PIZZA HUT</t>
         </is>
       </c>
     </row>
@@ -4907,7 +4907,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>ANDEN 3-4 MATRIZ PRINCIPAL</t>
+          <t>ANDEN 3-4 LOCALES GASTRONOMICOS</t>
         </is>
       </c>
     </row>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>ANDEN 3-4 RESTAURANTE</t>
+          <t>ANDEN 3-4 MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -4931,7 +4931,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>BAZAR GOURMET</t>
+          <t>ANDEN 3-4 RESTAURANTE</t>
         </is>
       </c>
     </row>
@@ -4943,7 +4943,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>DISTRITO DE LUJO</t>
+          <t>BAZAR GOURMET</t>
         </is>
       </c>
     </row>
@@ -4955,7 +4955,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>DL KENNEDY</t>
+          <t>DISTRITO DE LUJO</t>
         </is>
       </c>
     </row>
@@ -4967,7 +4967,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>LLENADO DE PILETA</t>
+          <t>DL KENNEDY</t>
         </is>
       </c>
     </row>
@@ -4979,7 +4979,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>PILETA CASCADA</t>
+          <t>LLENADO DE PILETA</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>SANDIA ANTIGUA</t>
+          <t>PILETA CASCADA</t>
         </is>
       </c>
     </row>
@@ -5003,19 +5003,19 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>SANDIA NUEVA</t>
+          <t>SANDIA ANTIGUA</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="B158" t="inlineStr">
         <is>
-          <t>PROVIDENCIA</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>CARMELA CARVAJAL</t>
+          <t>SANDIA NUEVA</t>
         </is>
       </c>
     </row>
@@ -5027,7 +5027,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>LASTARRIA</t>
+          <t>CARMELA CARVAJAL</t>
         </is>
       </c>
     </row>
@@ -5039,7 +5039,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>LICEO JUAN PABLO DUARTE</t>
+          <t>LASTARRIA</t>
         </is>
       </c>
     </row>
@@ -5051,19 +5051,19 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>LICEO N°7</t>
+          <t>LICEO JUAN PABLO DUARTE</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="B162" t="inlineStr">
         <is>
-          <t>RENCA</t>
+          <t>PROVIDENCIA</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>CAPITAN JOSÉ LUIS ARANDE</t>
+          <t>LICEO N°7</t>
         </is>
       </c>
     </row>
@@ -5075,7 +5075,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>JUAN DE ATALA HIRMAS</t>
+          <t>CAPITAN JOSÉ LUIS ARANDE</t>
         </is>
       </c>
     </row>
@@ -5087,19 +5087,19 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>REBECA MATTE BELLO</t>
+          <t>JUAN DE ATALA HIRMAS</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="B165" t="inlineStr">
         <is>
-          <t>UDD</t>
+          <t>RENCA</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS EDIFICIO ¨O¨</t>
+          <t>REBECA MATTE BELLO</t>
         </is>
       </c>
     </row>
@@ -5110,6 +5110,18 @@
         </is>
       </c>
       <c r="C166" t="inlineStr">
+        <is>
+          <t>SALA DE BOMBAS EDIFICIO ¨O¨</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>UDD</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
         <is>
           <t>SALA DE BOMBAS HONDURAS</t>
         </is>
@@ -5135,7 +5147,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="20">
-        <f>IFERROR(FILTER(Base1!B2:C166,Base1!B2:B166=Ingreso!C4),"")</f>
+        <f>IFERROR(FILTER(Base1!B2:C167,Base1!B2:B167=Ingreso!C4),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add multi-CC client contacts sheet for visit PDF emails.
Support roles like JO, environmental lead, and Linkes maintenance per client (e.g. MAE), with form auto-selection of TO/CC and firmante.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mantenimiento_wes/FORMULARIO_MANTENCION_WES_DIGITAL.xlsx
+++ b/mantenimiento_wes/FORMULARIO_MANTENCION_WES_DIGITAL.xlsx
@@ -10,15 +10,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ingreso" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formulario Visita" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base1" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base2" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base3" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base 4" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contactos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formulario Visita" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base2" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base3" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base 4" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Datos'!$B$1:$U$2000</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Contactos'!$A$1:$J$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -248,7 +250,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -291,6 +293,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -656,7 +661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -669,6 +674,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -683,6 +689,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -725,6 +732,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -753,6 +761,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
@@ -767,6 +776,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
@@ -777,8 +787,39 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Catálogos sincronizados: 2026-08-12 19:45 desde analisis_falla_google.xlsx · 28 clientes · 159 máquinas · 62 fallas</t>
-        </is>
+          <t>Catálogos sincronizados: 2026-08-17 18:29 desde analisis_falla_google.xlsx · 29 clientes · 171 máquinas · 62 fallas</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Contactos multi-CC: hoja Contactos. Completá Email / Rol (JO, Medio ambiente, Mantención Linkes). Firmante habitual = quien suele firmar. Enviar TO/CC = destino del PDF.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20">
+        <f>IFERROR(FILTER(Base3!B2:C63,Base3!B2:B63=Ingreso!C14),"")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -2491,6 +2532,939 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="B1" s="30" t="inlineStr">
+        <is>
+          <t>Sitio</t>
+        </is>
+      </c>
+      <c r="C1" s="30" t="inlineStr">
+        <is>
+          <t>Rol</t>
+        </is>
+      </c>
+      <c r="D1" s="30" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="E1" s="30" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="F1" s="30" t="inlineStr">
+        <is>
+          <t>Firmante habitual</t>
+        </is>
+      </c>
+      <c r="G1" s="30" t="inlineStr">
+        <is>
+          <t>Enviar TO</t>
+        </is>
+      </c>
+      <c r="H1" s="30" t="inlineStr">
+        <is>
+          <t>Enviar CC</t>
+        </is>
+      </c>
+      <c r="I1" s="30" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="J1" s="30" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>AEB</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr"/>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>Jefe de operaciones</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr"/>
+      <c r="E2" s="15" t="inlineStr"/>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I2" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J2" s="15" t="inlineStr">
+        <is>
+          <t>Reportar acta de visita</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>AEB</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr"/>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>Líder de medio ambiente</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr"/>
+      <c r="E3" s="15" t="inlineStr"/>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H3" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I3" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J3" s="15" t="inlineStr">
+        <is>
+          <t>Copia ambiental</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>AEB</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr"/>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Mantención Linkes</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr"/>
+      <c r="E4" s="15" t="inlineStr"/>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>Apoya la visita; suele firmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr"/>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Jefe de operaciones</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr"/>
+      <c r="E5" s="15" t="inlineStr"/>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I5" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J5" s="15" t="inlineStr">
+        <is>
+          <t>Reportar acta de visita</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr"/>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Líder de medio ambiente</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr"/>
+      <c r="E6" s="15" t="inlineStr"/>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I6" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J6" s="15" t="inlineStr">
+        <is>
+          <t>Copia ambiental</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr"/>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Mantención Linkes</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr"/>
+      <c r="E7" s="15" t="inlineStr"/>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I7" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J7" s="15" t="inlineStr">
+        <is>
+          <t>Apoya la visita; suele firmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>CUR</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr"/>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Jefe de operaciones</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr"/>
+      <c r="E8" s="15" t="inlineStr"/>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I8" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J8" s="15" t="inlineStr">
+        <is>
+          <t>Reportar acta de visita</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>CUR</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr"/>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>Líder de medio ambiente</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr"/>
+      <c r="E9" s="15" t="inlineStr"/>
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I9" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J9" s="15" t="inlineStr">
+        <is>
+          <t>Copia ambiental</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>CUR</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr"/>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Mantención Linkes</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr"/>
+      <c r="E10" s="15" t="inlineStr"/>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I10" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J10" s="15" t="inlineStr">
+        <is>
+          <t>Apoya la visita; suele firmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr"/>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>Jefe de operaciones</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr"/>
+      <c r="E11" s="15" t="inlineStr"/>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I11" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J11" s="15" t="inlineStr">
+        <is>
+          <t>Reportar acta de visita</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr"/>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>Líder de medio ambiente</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr"/>
+      <c r="E12" s="15" t="inlineStr"/>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I12" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J12" s="15" t="inlineStr">
+        <is>
+          <t>Copia ambiental</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr"/>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>Mantención Linkes</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr"/>
+      <c r="E13" s="15" t="inlineStr"/>
+      <c r="F13" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H13" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I13" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J13" s="15" t="inlineStr">
+        <is>
+          <t>Apoya la visita; suele firmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>MAM</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr"/>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>Jefe de operaciones</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr"/>
+      <c r="E14" s="15" t="inlineStr"/>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I14" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J14" s="15" t="inlineStr">
+        <is>
+          <t>Reportar acta de visita</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>MAM</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr"/>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>Líder de medio ambiente</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr"/>
+      <c r="E15" s="15" t="inlineStr"/>
+      <c r="F15" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I15" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J15" s="15" t="inlineStr">
+        <is>
+          <t>Copia ambiental</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>MAM</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr"/>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Mantención Linkes</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr"/>
+      <c r="E16" s="15" t="inlineStr"/>
+      <c r="F16" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I16" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J16" s="15" t="inlineStr">
+        <is>
+          <t>Apoya la visita; suele firmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>MAQ</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr"/>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>Jefe de operaciones</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr"/>
+      <c r="E17" s="15" t="inlineStr"/>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I17" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J17" s="15" t="inlineStr">
+        <is>
+          <t>Reportar acta de visita</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>MAQ</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr"/>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>Líder de medio ambiente</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr"/>
+      <c r="E18" s="15" t="inlineStr"/>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I18" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J18" s="15" t="inlineStr">
+        <is>
+          <t>Copia ambiental</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>MAQ</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr"/>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>Mantención Linkes</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr"/>
+      <c r="E19" s="15" t="inlineStr"/>
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H19" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I19" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J19" s="15" t="inlineStr">
+        <is>
+          <t>Apoya la visita; suele firmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>PAK</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr"/>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>Jefe de operaciones</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr"/>
+      <c r="E20" s="15" t="inlineStr"/>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G20" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I20" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J20" s="15" t="inlineStr">
+        <is>
+          <t>Reportar acta de visita</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>PAK</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr"/>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>Líder de medio ambiente</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr"/>
+      <c r="E21" s="15" t="inlineStr"/>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I21" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J21" s="15" t="inlineStr">
+        <is>
+          <t>Copia ambiental</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>PAK</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr"/>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>Mantención Linkes</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr"/>
+      <c r="E22" s="15" t="inlineStr"/>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H22" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I22" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J22" s="15" t="inlineStr">
+        <is>
+          <t>Apoya la visita; suele firmar</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J22"/>
+  <dataValidations count="4">
+    <dataValidation sqref="F2:F2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sí,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sí,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sí,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sí,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2539,7 +3513,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3110,13 +4084,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C160"/>
+  <dimension ref="B1:C172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -3246,48 +4220,48 @@
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>BUPA ANTOFGASTA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CALLE DE SERVICO</t>
+          <t>MEDIDOR PRINCIPAL SANITARIA</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>BUPA ANTOFGASTA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CLUB HOUSE</t>
+          <t>SALA DE BOMBA N°2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>BUPA ANTOFGASTA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>EDIFICIO DEPORTIVO</t>
+          <t>SALA DE BOMBA SEXTO PISO</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>BUPA ANTOFGASTA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>EDIFIO DEPORTIVO</t>
+          <t>SALA DE BOMBAS PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -3299,7 +4273,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>EQUITACION</t>
+          <t>CALLE DE SERVICO</t>
         </is>
       </c>
     </row>
@@ -3311,67 +4285,67 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>RAIMUNDO TUPPER</t>
+          <t>CANCHAS DE TENIS</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>COSTANERA</t>
+          <t>CLUB HOUSE</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ESTANQUE DE REUTILIZACION</t>
+          <t>EDIFICIO DEPORTIVO</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LAVADO AUTO SERVICIO NORTE</t>
+          <t>EDIFIO DEPORTIVO</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>LAVADO AUTO SERVICIO SUR</t>
+          <t>EQUITACION</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>CDUC</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>LAVADO AUTOMATICO NORTE</t>
+          <t>RAIMUNDO TUPPER</t>
         </is>
       </c>
     </row>
@@ -3383,7 +4357,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>LAVADO AUTOMATICO SUR</t>
+          <t>COSTANERA</t>
         </is>
       </c>
     </row>
@@ -3395,7 +4369,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>ESTANQUE DE REUTILIZACION</t>
         </is>
       </c>
     </row>
@@ -3407,7 +4381,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>OFICINA ADMIN</t>
+          <t>LAVADO AUTO SERVICIO NORTE</t>
         </is>
       </c>
     </row>
@@ -3419,7 +4393,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PRONTO BAÑO</t>
+          <t>LAVADO AUTO SERVICIO SUR</t>
         </is>
       </c>
     </row>
@@ -3431,7 +4405,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PRONTO TIENDA</t>
+          <t>LAVADO AUTOMATICO NORTE</t>
         </is>
       </c>
     </row>
@@ -3443,67 +4417,67 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>RIEGO</t>
+          <t>LAVADO AUTOMATICO SUR</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>COMPLEJO EDUCACIONAL CONSOLIDADA</t>
+          <t>MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ESCUELA ANDES DEL SUR</t>
+          <t>OFICINA ADMIN</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ESCUELA GABRIELA</t>
+          <t>PRONTO BAÑO</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ESCUELA JUAN MACKENNA</t>
+          <t>PRONTO TIENDA</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ESCUELA LOS ANDES</t>
+          <t>RIEGO</t>
         </is>
       </c>
     </row>
@@ -3515,7 +4489,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ESCUELA LUIS MATTE LARRAIN</t>
+          <t>COMPLEJO EDUCACIONAL CONSOLIDADA</t>
         </is>
       </c>
     </row>
@@ -3527,7 +4501,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ESCUELA PADRE HURTADO</t>
+          <t>ESCUELA ANDES DEL SUR</t>
         </is>
       </c>
     </row>
@@ -3539,7 +4513,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ESCUELA VILLA INDEPENDENCIA</t>
+          <t>ESCUELA GABRIELA</t>
         </is>
       </c>
     </row>
@@ -3551,7 +4525,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ESCULA NONATO COO</t>
+          <t>ESCUELA JUAN MACKENNA</t>
         </is>
       </c>
     </row>
@@ -3563,7 +4537,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LICEO CHILOE</t>
+          <t>ESCUELA LOS ANDES</t>
         </is>
       </c>
     </row>
@@ -3575,67 +4549,67 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>LICEO MAIPO</t>
+          <t>ESCUELA LUIS MATTE LARRAIN</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ALICURA</t>
+          <t>ESCUELA PADRE HURTADO</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ANTONIO HERMIDA FABRES</t>
+          <t>ESCUELA VILLA INDEPENDENCIA</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CARLOS FERNANDEZ PEÑA</t>
+          <t>ESCULA NONATO COO</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CENTRO EDUCACIONAL EDUARDO DE LA BARRA</t>
+          <t>LICEO CHILOE</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>CENTRO EDUCACIONAL VALLE HERMOSO</t>
+          <t>LICEO MAIPO</t>
         </is>
       </c>
     </row>
@@ -3647,7 +4621,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ERASMO ESCALA</t>
+          <t>ALICURA</t>
         </is>
       </c>
     </row>
@@ -3659,7 +4633,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ESCUELA ESPECIAL PONTÍFICE JUAN PABLO II</t>
+          <t>ANTONIO HERMIDA FABRES</t>
         </is>
       </c>
     </row>
@@ -3671,7 +4645,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ESCUELA LUIS ARRIETA CAÑAS</t>
+          <t>CARLOS FERNANDEZ PEÑA</t>
         </is>
       </c>
     </row>
@@ -3683,7 +4657,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ESCUELA UNIÓN NACIONAL ÁRABE</t>
+          <t>CENTRO EDUCACIONAL EDUARDO DE LA BARRA</t>
         </is>
       </c>
     </row>
@@ -3695,7 +4669,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>JUAN BAUTISTA PASTENE</t>
+          <t>CENTRO EDUCACIONAL VALLE HERMOSO</t>
         </is>
       </c>
     </row>
@@ -3707,7 +4681,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>LIKANKURA</t>
+          <t>ERASMO ESCALA</t>
         </is>
       </c>
     </row>
@@ -3719,7 +4693,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>MATILDE HUICI NAVAS</t>
+          <t>ESCUELA ESPECIAL PONTÍFICE JUAN PABLO II</t>
         </is>
       </c>
     </row>
@@ -3731,7 +4705,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>SANTA MARIA</t>
+          <t>ESCUELA LUIS ARRIETA CAÑAS</t>
         </is>
       </c>
     </row>
@@ -3743,91 +4717,91 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>TOBALABA</t>
+          <t>ESCUELA UNIÓN NACIONAL ÁRABE</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" t="inlineStr">
         <is>
-          <t>CUR</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ANILLO NORTE</t>
+          <t>JUAN BAUTISTA PASTENE</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" t="inlineStr">
         <is>
-          <t>CUR</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ANILLO SUR</t>
+          <t>LIKANKURA</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
-          <t>CUR</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>BAÑOS</t>
+          <t>MATILDE HUICI NAVAS</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" t="inlineStr">
         <is>
-          <t>CUR</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>SANTA MARIA</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>LO BOZA - EDIFICIO PRINCIPAL CASINO</t>
+          <t>TOBALABA</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="B58" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>CUR</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>LO BOZA - LAVADO DE VEHICULOS</t>
+          <t>ANILLO NORTE</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>CUR</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>LO BOZA - POZO DE LAVADO DE VEHICULO</t>
+          <t>ANILLO SUR</t>
         </is>
       </c>
     </row>
@@ -3839,7 +4813,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>LO BOZA - REUTILIZACION</t>
+          <t>LO BOZA - EDIFICIO PRINCIPAL CASINO</t>
         </is>
       </c>
     </row>
@@ -3851,7 +4825,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>LO BOZA - SALA DE IMPULSION</t>
+          <t>LO BOZA - LAVADO DE VEHICULOS</t>
         </is>
       </c>
     </row>
@@ -3863,7 +4837,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>OPEN PLAZA - MATRIZ PRINCIPAL</t>
+          <t>LO BOZA - POZO DE LAVADO DE VEHICULO</t>
         </is>
       </c>
     </row>
@@ -3875,7 +4849,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>PRONTO BAÑO</t>
+          <t>LO BOZA - REUTILIZACION</t>
         </is>
       </c>
     </row>
@@ -3887,7 +4861,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>QUILICURA - CAMARINES</t>
+          <t>LO BOZA - SALA DE IMPULSION</t>
         </is>
       </c>
     </row>
@@ -3899,7 +4873,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>QUILICURA - CASINO</t>
+          <t>OPEN PLAZA - MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -3911,7 +4885,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>QUILICURA - DERCOMAQ</t>
+          <t>PRONTO BAÑO</t>
         </is>
       </c>
     </row>
@@ -3923,7 +4897,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>QUILICURA - EDIFICIO JCB</t>
+          <t>QUILICURA - CAMARINES</t>
         </is>
       </c>
     </row>
@@ -3935,7 +4909,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>QUILICURA - LAVADO DE MAQUINA</t>
+          <t>QUILICURA - CASINO</t>
         </is>
       </c>
     </row>
@@ -3947,7 +4921,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>QUILICURA - MATRIZ PRINCIPAL</t>
+          <t>QUILICURA - DERCOMAQ</t>
         </is>
       </c>
     </row>
@@ -3959,67 +4933,67 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>QUILICURA - PRODERCO</t>
+          <t>QUILICURA - EDIFICIO JCB</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="B71" t="inlineStr">
         <is>
-          <t>ESTADIO ISRAELITA</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>MATRIS CHESTERTON</t>
+          <t>QUILICURA - LAVADO DE MAQUINA</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="B72" t="inlineStr">
         <is>
-          <t>ESTADIO ISRAELITA</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>MATRIZ AV LAS CONDES</t>
+          <t>QUILICURA - MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="B73" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>ETAPA 1,2,3 Y 4</t>
+          <t>QUILICURA - PRODERCO</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="B74" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>ESTADIO ISRAELITA</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ETAPA 5</t>
+          <t>MATRIS CHESTERTON</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="B75" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>ESTADIO ISRAELITA</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>MATRIS ESVAL</t>
+          <t>MATRIZ AV LAS CONDES</t>
         </is>
       </c>
     </row>
@@ -4031,103 +5005,103 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>RIEGO</t>
+          <t>ESTANQUE INFERIOR</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="B77" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>CDP PUENTE ALTO</t>
+          <t>ETAPA 1</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="B78" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>COLINA 1</t>
+          <t>ETAPA 1,2,3 Y 4</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="B79" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>COLINA 2 RED SUR</t>
+          <t>ETAPA 1-4</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="B80" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>COLINA 2 REDIMPULSION</t>
+          <t>ETAPA 2</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="B81" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>CPA MODULO</t>
+          <t>ETAPA 3</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="B82" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>CPA OVALO</t>
+          <t>ETAPA 5</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="B83" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>CPF SAN MIGUEL MATRIZ PRINCIPAL</t>
+          <t>MATRIS ESVAL</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="B84" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>CPF SAN MIGUEL SALA IMPULSION</t>
+          <t>RIEGO LLENADO DE ESTANQUE ESVAL</t>
         </is>
       </c>
     </row>
@@ -4139,7 +5113,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ESC. EL BOSQUE ADMINISTRACION</t>
+          <t>CDP PUENTE ALTO</t>
         </is>
       </c>
     </row>
@@ -4151,7 +5125,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>ESC. EL BOSQUE GENCHI ACADEMIA</t>
+          <t>COLINA 1</t>
         </is>
       </c>
     </row>
@@ -4163,7 +5137,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ESC. OF ARTEMIO</t>
+          <t>COLINA 2 RED SUR</t>
         </is>
       </c>
     </row>
@@ -4175,7 +5149,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ESC. OF CARMEN</t>
+          <t>COLINA 2 REDIMPULSION</t>
         </is>
       </c>
     </row>
@@ -4187,7 +5161,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>ESCUELA ANDES DEL SUR</t>
+          <t>CPA MODULO</t>
         </is>
       </c>
     </row>
@@ -4199,7 +5173,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>ESFORPEN BOSQUE ADMINISTRACION</t>
+          <t>CPA OVALO</t>
         </is>
       </c>
     </row>
@@ -4211,7 +5185,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>ESFORPEN BOSQUE GENCHI SIMULACION</t>
+          <t>CPF SAN MIGUEL MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -4223,7 +5197,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>MONITOREO MATRIZ PRINCIPAL MODULO</t>
+          <t>CPF SAN MIGUEL SALA IMPULSION</t>
         </is>
       </c>
     </row>
@@ -4235,511 +5209,511 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>MONITOREO MATRIZ PRINCIPAL OVALO</t>
+          <t>ESC. EL BOSQUE ADMINISTRACION</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="B94" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>AGUA BLANDA</t>
+          <t>ESC. EL BOSQUE GENCHI ACADEMIA</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="B95" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>INTERCAMBIADOR 1</t>
+          <t>ESC. OF ARTEMIO</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="B96" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>INTERCAMBIADOR 2</t>
+          <t>ESC. OF CARMEN</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="B97" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>ESCUELA ANDES DEL SUR</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="B98" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>RETORNO OSMOSIS</t>
+          <t>ESFORPEN BOSQUE ADMINISTRACION</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="B99" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>SALIDA OSMOSIS</t>
+          <t>ESFORPEN BOSQUE GENCHI SIMULACION</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="B100" t="inlineStr">
         <is>
-          <t>LA FLORIDA</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>LICEO ALTO CORDILLERA</t>
+          <t>MONITOREO MATRIZ PRINCIPAL MODULO</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="B101" t="inlineStr">
         <is>
-          <t>LA REINA</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>EUGENIO MARIA DE HOSTOS</t>
+          <t>MONITOREO MATRIZ PRINCIPAL OVALO</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>LAS CONDES</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>FLEMING</t>
+          <t>AGUA BLANDA</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="B103" t="inlineStr">
         <is>
-          <t>LAS CONDES</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>JUAN PABLO II</t>
+          <t>INTERCAMBIADOR 1</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
-          <t>LAS CONDES</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>LIKANKURA</t>
+          <t>INTERCAMBIADOR 2</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="B105" t="inlineStr">
         <is>
-          <t>LO VALLEDOR</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>BARRIO NORTE</t>
+          <t>MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="B106" t="inlineStr">
         <is>
-          <t>LO VALLEDOR</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>POZO 1</t>
+          <t>RETORNO OSMOSIS</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="B107" t="inlineStr">
         <is>
-          <t>LO VALLEDOR</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>PUERTA 1</t>
+          <t>SALIDA OSMOSIS</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="B108" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>LA FLORIDA</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>CASINO</t>
+          <t>LICEO ALTO CORDILLERA</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>LA REINA</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>ESTANQUE CISTERNA</t>
+          <t>EUGENIO MARIA DE HOSTOS</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="B110" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>LAS CONDES</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>SAN NICOLAS</t>
+          <t>FLEMING</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="B111" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>LAS CONDES</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>URETA COX</t>
+          <t>JUAN PABLO II</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="B112" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>LAS CONDES</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>BAÑO GUARDIAS</t>
+          <t>LIKANKURA</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="B113" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>LO VALLEDOR</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
+          <t>BARRIO NORTE</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="B114" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>LO VALLEDOR</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>ESTANQUE NORTE LOCALES</t>
+          <t>POZO 1</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="B115" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>LO VALLEDOR</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>ESTANQUE SUR ABASTECIMIENTO</t>
+          <t>PUERTA 1</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="B116" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>KFC</t>
+          <t>CASINO</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="B117" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>PIZZA HUT</t>
+          <t>ESTANQUE CISTERNA</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="B118" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>MATRIZ BOULEVARD PASILLO TECNICO</t>
+          <t>SAN NICOLAS</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="B119" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>MATRIZ SALIDA DE EMERGENCIA PASILLO N°1 ARROW</t>
+          <t>URETA COX</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="B120" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>PLACA BANCARIA</t>
+          <t>BAÑO GUARDIAS</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="B121" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS FALABELLA</t>
+          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="B122" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS RIPLEY</t>
+          <t>ESTANQUE NORTE LOCALES</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="B123" t="inlineStr">
         <is>
-          <t>MAQ</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>ALIMENTACION DE BAÑOS</t>
+          <t>KFC</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="B124" t="inlineStr">
         <is>
-          <t>MAQ</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>PIZZA HUT</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="B125" t="inlineStr">
         <is>
-          <t>MAQ</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>RED DE INCENDIO</t>
+          <t>SALA DE BOMBAS ESTANQUE SUR</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="B126" t="inlineStr">
         <is>
-          <t>MOLYMET</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>CASA DE CAMBIO</t>
+          <t>MATRIZ BOULEVARD PASILLO TECNICO</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="B127" t="inlineStr">
         <is>
-          <t>MOLYMET</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>RIEGO</t>
+          <t>MATRIZ SALIDA DE EMERGENCIA PASILLO N°1 ARROW</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="B128" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>CANCHA</t>
+          <t>PLACA BANCARIA</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="B129" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>CONTROL NIDO</t>
+          <t>SALA DE BOMBAS FALABELLA</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="B130" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ELEMENTARY</t>
+          <t>SALA DE BOMBAS RIPLEY</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="B131" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>MAQ</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ESTANQUE B</t>
+          <t>ALIMENTACION DE BAÑOS</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="B132" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>MAQ</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>ESTANQUE C</t>
+          <t>MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="B133" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>MAQ</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>HIGH SCHOOL</t>
+          <t>RED DE INCENDIO</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="B134" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>MOLYMET</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>PISCINA</t>
+          <t>CASA DE CAMBIO</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="B135" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>MOLYMET</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>POZO PROFUNDO</t>
+          <t>RIEGO</t>
         </is>
       </c>
     </row>
@@ -4751,151 +5725,151 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>TEATRO</t>
+          <t>CANCHA</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="B137" t="inlineStr">
         <is>
-          <t>PAE</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
+          <t>CONTROL NIDO</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="B138" t="inlineStr">
         <is>
-          <t>PAE</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>ESTANQUE NORTE LOCALES</t>
+          <t>ELEMENTARY</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="B139" t="inlineStr">
         <is>
-          <t>PAE</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>KFC</t>
+          <t>ESTANQUE B</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="B140" t="inlineStr">
         <is>
-          <t>PAE</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>PIZZA HUT</t>
+          <t>ESTANQUE C</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="B141" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>ANDEN 3-4 LOCALES GASTRONOMICOS</t>
+          <t>HIGH SCHOOL</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="B142" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>ANDEN 3-4 MATRIZ PRINCIPAL</t>
+          <t>PISCINA</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="B143" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>ANDEN 3-4 RESTAURANTE</t>
+          <t>POZO PROFUNDO</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="B144" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>BAZAR GOURMET</t>
+          <t>TEATRO</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="B145" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>BAÑO DAMAS</t>
+          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="B146" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>BAÑO VARONES</t>
+          <t>ESTANQUE NORTE LOCALES</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="B147" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>DISTRITO DE LUJO</t>
+          <t>KFC</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="B148" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>DL KENNEDY</t>
+          <t>PIZZA HUT</t>
         </is>
       </c>
     </row>
@@ -4907,7 +5881,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>LLENADO DE PILETA</t>
+          <t>ANDEN 3-4 LOCALES GASTRONOMICOS</t>
         </is>
       </c>
     </row>
@@ -4919,7 +5893,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>PILETA CASCADA</t>
+          <t>ANDEN 3-4 MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -4931,7 +5905,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>SANDIA ANTIGUA</t>
+          <t>ANDEN 3-4 RESTAURANTE</t>
         </is>
       </c>
     </row>
@@ -4943,101 +5917,245 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>SANDIA NUEVA</t>
+          <t>BAZAR GOURMET</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="B153" t="inlineStr">
         <is>
-          <t>PROVIDENCIA</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>ARTURO ALESSANDRI PALMA</t>
+          <t>DISTRITO DE LUJO</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="B154" t="inlineStr">
         <is>
-          <t>PROVIDENCIA</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>CARMELA CARVAJAL</t>
+          <t>DL KENNEDY</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="B155" t="inlineStr">
         <is>
-          <t>PROVIDENCIA</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>LASTARRIA</t>
+          <t>LLENADO DE PILETA</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="B156" t="inlineStr">
         <is>
-          <t>RENCA</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>CAPITAN JOSÉ LUIS ARANDE</t>
+          <t>PILETA CASCADA</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="B157" t="inlineStr">
         <is>
-          <t>RENCA</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>JUAN DE ATALA HIRMAS</t>
+          <t>SANDIA ANTIGUA</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="B158" t="inlineStr">
         <is>
-          <t>RENCA</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>REBECA MATTE BELLO</t>
+          <t>SANDIA NUEVA</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="B159" t="inlineStr">
         <is>
-          <t>UDD</t>
+          <t>PROVIDENCIA</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS EDIFICIO ¨O¨</t>
+          <t>CARMELA CARVAJAL</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="B160" t="inlineStr">
         <is>
+          <t>PROVIDENCIA</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>LASTARRIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>PROVIDENCIA</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>LICEO JUAN PABLO DUARTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>PROVIDENCIA</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>LICEO N°7</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>CAPITAN JOSÉ LUIS ARANDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>ESCUELA LO VELZAQUEZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>GYM MUNICIPAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>INSTITUTO CUMBRE DE CONDORES ORIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>INSTITUTO CUMBRE DE CONDORES PONIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>JUAN DE ATALA HIRMAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>PISCINA MUNICIPAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>REBECA MATTE BELLO</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="B171" t="inlineStr">
+        <is>
           <t>UDD</t>
         </is>
       </c>
-      <c r="C160" t="inlineStr">
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>SALA DE BOMBAS EDIFICIO ¨O¨</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>UDD</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
         <is>
           <t>SALA DE BOMBAS HONDURAS</t>
         </is>
@@ -5048,7 +6166,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5063,7 +6181,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="20">
-        <f>IFERROR(FILTER(Base1!B2:C160,Base1!B2:B160=Ingreso!C4),"")</f>
+        <f>IFERROR(FILTER(Base1!B2:C172,Base1!B2:B172=Ingreso!C4),"")</f>
         <v/>
       </c>
     </row>
@@ -5072,7 +6190,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5844,28 +6962,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="20">
-        <f>IFERROR(FILTER(Base3!B2:C63,Base3!B2:B63=Ingreso!C14),"")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Unify visit-form emails on CONTACTOS_ENVIOS_ACTAS only.
Drop the duplicate Contactos sheet seed; sync TO/CC from the official
Drive workbook so MAE (and others) stop picking the wrong Excel.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mantenimiento_wes/FORMULARIO_MANTENCION_WES_DIGITAL.xlsx
+++ b/mantenimiento_wes/FORMULARIO_MANTENCION_WES_DIGITAL.xlsx
@@ -20,7 +20,6 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Datos'!$B$1:$U$2000</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Contactos'!$A$1:$J$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -31,7 +30,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -96,6 +95,11 @@
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00666666"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="7">
@@ -250,7 +254,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -296,6 +300,8 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -674,7 +680,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -689,7 +694,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -732,7 +736,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -761,7 +764,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
@@ -776,7 +778,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
@@ -2532,929 +2533,82 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="30" t="inlineStr">
-        <is>
-          <t>Cliente</t>
-        </is>
-      </c>
-      <c r="B1" s="30" t="inlineStr">
-        <is>
-          <t>Sitio</t>
-        </is>
-      </c>
-      <c r="C1" s="30" t="inlineStr">
-        <is>
-          <t>Rol</t>
-        </is>
-      </c>
-      <c r="D1" s="30" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="E1" s="30" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="F1" s="30" t="inlineStr">
-        <is>
-          <t>Firmante habitual</t>
-        </is>
-      </c>
-      <c r="G1" s="30" t="inlineStr">
-        <is>
-          <t>Enviar TO</t>
-        </is>
-      </c>
-      <c r="H1" s="30" t="inlineStr">
-        <is>
-          <t>Enviar CC</t>
-        </is>
-      </c>
-      <c r="I1" s="30" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="J1" s="30" t="inlineStr">
-        <is>
-          <t>Notas</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="15" t="inlineStr">
-        <is>
-          <t>AEB</t>
-        </is>
-      </c>
-      <c r="B2" s="15" t="inlineStr"/>
-      <c r="C2" s="15" t="inlineStr">
-        <is>
-          <t>Jefe de operaciones</t>
-        </is>
-      </c>
-      <c r="D2" s="15" t="inlineStr"/>
-      <c r="E2" s="15" t="inlineStr"/>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J2" s="15" t="inlineStr">
-        <is>
-          <t>Reportar acta de visita</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>AEB</t>
-        </is>
-      </c>
-      <c r="B3" s="15" t="inlineStr"/>
-      <c r="C3" s="15" t="inlineStr">
-        <is>
-          <t>Líder de medio ambiente</t>
-        </is>
-      </c>
-      <c r="D3" s="15" t="inlineStr"/>
-      <c r="E3" s="15" t="inlineStr"/>
-      <c r="F3" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G3" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H3" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I3" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J3" s="15" t="inlineStr">
-        <is>
-          <t>Copia ambiental</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>AEB</t>
-        </is>
-      </c>
-      <c r="B4" s="15" t="inlineStr"/>
-      <c r="C4" s="15" t="inlineStr">
-        <is>
-          <t>Mantención Linkes</t>
-        </is>
-      </c>
-      <c r="D4" s="15" t="inlineStr"/>
-      <c r="E4" s="15" t="inlineStr"/>
-      <c r="F4" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G4" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="H4" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I4" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J4" s="15" t="inlineStr">
-        <is>
-          <t>Apoya la visita; suele firmar</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>BOM</t>
-        </is>
-      </c>
-      <c r="B5" s="15" t="inlineStr"/>
-      <c r="C5" s="15" t="inlineStr">
-        <is>
-          <t>Jefe de operaciones</t>
-        </is>
-      </c>
-      <c r="D5" s="15" t="inlineStr"/>
-      <c r="E5" s="15" t="inlineStr"/>
-      <c r="F5" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G5" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H5" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I5" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J5" s="15" t="inlineStr">
-        <is>
-          <t>Reportar acta de visita</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>BOM</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="inlineStr"/>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>Líder de medio ambiente</t>
-        </is>
-      </c>
-      <c r="D6" s="15" t="inlineStr"/>
-      <c r="E6" s="15" t="inlineStr"/>
-      <c r="F6" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G6" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H6" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I6" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J6" s="15" t="inlineStr">
-        <is>
-          <t>Copia ambiental</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>BOM</t>
-        </is>
-      </c>
-      <c r="B7" s="15" t="inlineStr"/>
-      <c r="C7" s="15" t="inlineStr">
-        <is>
-          <t>Mantención Linkes</t>
-        </is>
-      </c>
-      <c r="D7" s="15" t="inlineStr"/>
-      <c r="E7" s="15" t="inlineStr"/>
-      <c r="F7" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G7" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="H7" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I7" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J7" s="15" t="inlineStr">
-        <is>
-          <t>Apoya la visita; suele firmar</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t>CUR</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="inlineStr"/>
-      <c r="C8" s="15" t="inlineStr">
-        <is>
-          <t>Jefe de operaciones</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="inlineStr"/>
-      <c r="E8" s="15" t="inlineStr"/>
-      <c r="F8" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G8" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H8" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I8" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J8" s="15" t="inlineStr">
-        <is>
-          <t>Reportar acta de visita</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>CUR</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="inlineStr"/>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>Líder de medio ambiente</t>
-        </is>
-      </c>
-      <c r="D9" s="15" t="inlineStr"/>
-      <c r="E9" s="15" t="inlineStr"/>
-      <c r="F9" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G9" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H9" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I9" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J9" s="15" t="inlineStr">
-        <is>
-          <t>Copia ambiental</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="15" t="inlineStr">
-        <is>
-          <t>CUR</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr"/>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>Mantención Linkes</t>
-        </is>
-      </c>
-      <c r="D10" s="15" t="inlineStr"/>
-      <c r="E10" s="15" t="inlineStr"/>
-      <c r="F10" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G10" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="H10" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I10" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J10" s="15" t="inlineStr">
-        <is>
-          <t>Apoya la visita; suele firmar</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="15" t="inlineStr">
-        <is>
-          <t>MAE</t>
-        </is>
-      </c>
-      <c r="B11" s="15" t="inlineStr"/>
-      <c r="C11" s="15" t="inlineStr">
-        <is>
-          <t>Jefe de operaciones</t>
-        </is>
-      </c>
-      <c r="D11" s="15" t="inlineStr"/>
-      <c r="E11" s="15" t="inlineStr"/>
-      <c r="F11" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G11" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H11" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I11" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J11" s="15" t="inlineStr">
-        <is>
-          <t>Reportar acta de visita</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>MAE</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="inlineStr"/>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>Líder de medio ambiente</t>
-        </is>
-      </c>
-      <c r="D12" s="15" t="inlineStr"/>
-      <c r="E12" s="15" t="inlineStr"/>
-      <c r="F12" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G12" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H12" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I12" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J12" s="15" t="inlineStr">
-        <is>
-          <t>Copia ambiental</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>MAE</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="inlineStr"/>
-      <c r="C13" s="15" t="inlineStr">
-        <is>
-          <t>Mantención Linkes</t>
-        </is>
-      </c>
-      <c r="D13" s="15" t="inlineStr"/>
-      <c r="E13" s="15" t="inlineStr"/>
-      <c r="F13" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G13" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="H13" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I13" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J13" s="15" t="inlineStr">
-        <is>
-          <t>Apoya la visita; suele firmar</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>MAM</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="inlineStr"/>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>Jefe de operaciones</t>
-        </is>
-      </c>
-      <c r="D14" s="15" t="inlineStr"/>
-      <c r="E14" s="15" t="inlineStr"/>
-      <c r="F14" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G14" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H14" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I14" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J14" s="15" t="inlineStr">
-        <is>
-          <t>Reportar acta de visita</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>MAM</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="inlineStr"/>
-      <c r="C15" s="15" t="inlineStr">
-        <is>
-          <t>Líder de medio ambiente</t>
-        </is>
-      </c>
-      <c r="D15" s="15" t="inlineStr"/>
-      <c r="E15" s="15" t="inlineStr"/>
-      <c r="F15" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G15" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H15" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I15" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J15" s="15" t="inlineStr">
-        <is>
-          <t>Copia ambiental</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>MAM</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="inlineStr"/>
-      <c r="C16" s="15" t="inlineStr">
-        <is>
-          <t>Mantención Linkes</t>
-        </is>
-      </c>
-      <c r="D16" s="15" t="inlineStr"/>
-      <c r="E16" s="15" t="inlineStr"/>
-      <c r="F16" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G16" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="H16" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I16" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J16" s="15" t="inlineStr">
-        <is>
-          <t>Apoya la visita; suele firmar</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>MAQ</t>
-        </is>
-      </c>
-      <c r="B17" s="15" t="inlineStr"/>
-      <c r="C17" s="15" t="inlineStr">
-        <is>
-          <t>Jefe de operaciones</t>
-        </is>
-      </c>
-      <c r="D17" s="15" t="inlineStr"/>
-      <c r="E17" s="15" t="inlineStr"/>
-      <c r="F17" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G17" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H17" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I17" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J17" s="15" t="inlineStr">
-        <is>
-          <t>Reportar acta de visita</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="15" t="inlineStr">
-        <is>
-          <t>MAQ</t>
-        </is>
-      </c>
-      <c r="B18" s="15" t="inlineStr"/>
-      <c r="C18" s="15" t="inlineStr">
-        <is>
-          <t>Líder de medio ambiente</t>
-        </is>
-      </c>
-      <c r="D18" s="15" t="inlineStr"/>
-      <c r="E18" s="15" t="inlineStr"/>
-      <c r="F18" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G18" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H18" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I18" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J18" s="15" t="inlineStr">
-        <is>
-          <t>Copia ambiental</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>MAQ</t>
-        </is>
-      </c>
-      <c r="B19" s="15" t="inlineStr"/>
-      <c r="C19" s="15" t="inlineStr">
-        <is>
-          <t>Mantención Linkes</t>
-        </is>
-      </c>
-      <c r="D19" s="15" t="inlineStr"/>
-      <c r="E19" s="15" t="inlineStr"/>
-      <c r="F19" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G19" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="H19" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I19" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J19" s="15" t="inlineStr">
-        <is>
-          <t>Apoya la visita; suele firmar</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="15" t="inlineStr">
-        <is>
-          <t>PAK</t>
-        </is>
-      </c>
-      <c r="B20" s="15" t="inlineStr"/>
-      <c r="C20" s="15" t="inlineStr">
-        <is>
-          <t>Jefe de operaciones</t>
-        </is>
-      </c>
-      <c r="D20" s="15" t="inlineStr"/>
-      <c r="E20" s="15" t="inlineStr"/>
-      <c r="F20" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G20" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H20" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I20" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J20" s="15" t="inlineStr">
-        <is>
-          <t>Reportar acta de visita</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>PAK</t>
-        </is>
-      </c>
-      <c r="B21" s="15" t="inlineStr"/>
-      <c r="C21" s="15" t="inlineStr">
-        <is>
-          <t>Líder de medio ambiente</t>
-        </is>
-      </c>
-      <c r="D21" s="15" t="inlineStr"/>
-      <c r="E21" s="15" t="inlineStr"/>
-      <c r="F21" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G21" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H21" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I21" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J21" s="15" t="inlineStr">
-        <is>
-          <t>Copia ambiental</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>PAK</t>
-        </is>
-      </c>
-      <c r="B22" s="15" t="inlineStr"/>
-      <c r="C22" s="15" t="inlineStr">
-        <is>
-          <t>Mantención Linkes</t>
-        </is>
-      </c>
-      <c r="D22" s="15" t="inlineStr"/>
-      <c r="E22" s="15" t="inlineStr"/>
-      <c r="F22" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G22" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="H22" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I22" s="15" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J22" s="15" t="inlineStr">
-        <is>
-          <t>Apoya la visita; suele firmar</t>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>NO EDITAR CONTACTOS AQUÍ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="32" t="inlineStr">
+        <is>
+          <t>Fuente ÚNICA de correos:</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>CONTACTOS_ENVIOS_ACTAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>G:\Mi unidad\Agente WES\wes-scripts\mantenimiento wes\CONTACTOS_ENVIOS_ACTAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/spreadsheets/d/1Tpjm1eXRXKuKvxachtbYVr9503wICJdsYDTjkbm__o8/edit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="32" t="n"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="32" t="inlineStr">
+        <is>
+          <t>Columnas: Cliente | Máquina | Rol | Nombre | Cargo | Email | Actualizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="32" t="inlineStr">
+        <is>
+          <t>Roles: general=TO · CC/punto=CC (Máquina vacía = todo el cliente)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="32" t="inlineStr">
+        <is>
+          <t>Sincronizar al formulario: python contactos_cliente.py --desde-drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="32" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="32" t="inlineStr">
+        <is>
+          <t>Esta hoja queda solo como aviso para evitar confusión con planillas duplicadas.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J22"/>
-  <dataValidations count="4">
-    <dataValidation sqref="F2:F2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Sí,No"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G2:G2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Sí,No"</formula1>
-    </dataValidation>
-    <dataValidation sqref="H2:H2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Sí,No"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I2:I2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Sí,No"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix form machine list: use Clientes_catalogo, not Base1.
RENCA and other points were stale because sync read Registro Base1
(old names). Dropdowns now come from CONTACTOS_ENVIOS_ACTAS!Clientes_catalogo
so they match email contacts (ICCO/ICCP, GIMNASIO, etc.).

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mantenimiento_wes/FORMULARIO_MANTENCION_WES_DIGITAL.xlsx
+++ b/mantenimiento_wes/FORMULARIO_MANTENCION_WES_DIGITAL.xlsx
@@ -788,7 +788,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Catálogos sincronizados: 2026-08-17 19:27 desde analisis_falla_google.xlsx · 29 clientes · 171 máquinas · 62 fallas</t>
+          <t>Catálogos sync 2026-08-17 20:17: puntos desde CONTACTOS_ENVIOS_ACTAS!Clientes_catalogo · 29 clientes · 155 máquinas · fallas desde Registro Base3 (62)</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C172"/>
+  <dimension ref="B1:C156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MATRIZ A.A</t>
+          <t>MATRIZ PRIMER PISO</t>
         </is>
       </c>
     </row>
@@ -3283,19 +3283,19 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MATRIZ PRIMER PISO</t>
+          <t>MATRIZ RIEGO PLAZA</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>AEB</t>
+          <t>AGUNSA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MATRIZ RIEGO PLAZA</t>
+          <t>DEPOSITO</t>
         </is>
       </c>
     </row>
@@ -3307,7 +3307,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DEPOSITO</t>
+          <t>INTERMODAL</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>EDIFICIO DEPORTIVO</t>
+          <t>EQUITACION</t>
         </is>
       </c>
     </row>
@@ -3475,31 +3475,31 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>EDIFIO DEPORTIVO</t>
+          <t>RAIMUNDO TUPPER</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>EQUITACION</t>
+          <t>COSTANERA</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>CDUC</t>
+          <t>COPEC</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>RAIMUNDO TUPPER</t>
+          <t>ESTANQUE DE REUTILIZACION</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>COSTANERA</t>
+          <t>LAVADO AUTO SERVICIO NORTE</t>
         </is>
       </c>
     </row>
@@ -3523,7 +3523,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ESTANQUE DE REUTILIZACION</t>
+          <t>LAVADO AUTO SERVICIO SUR</t>
         </is>
       </c>
     </row>
@@ -3535,7 +3535,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>LAVADO AUTO SERVICIO NORTE</t>
+          <t>LAVADO AUTOMATICO NORTE</t>
         </is>
       </c>
     </row>
@@ -3547,7 +3547,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LAVADO AUTO SERVICIO SUR</t>
+          <t>LAVADO AUTOMATICO SUR</t>
         </is>
       </c>
     </row>
@@ -3559,7 +3559,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LAVADO AUTOMATICO NORTE</t>
+          <t>MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>LAVADO AUTOMATICO SUR</t>
+          <t>OFICINA ADMIN</t>
         </is>
       </c>
     </row>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>PRONTO BAÑO</t>
         </is>
       </c>
     </row>
@@ -3595,7 +3595,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>OFICINA ADMIN</t>
+          <t>PRONTO TIENDA</t>
         </is>
       </c>
     </row>
@@ -3607,31 +3607,31 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PRONTO BAÑO</t>
+          <t>RIEGO</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PRONTO TIENDA</t>
+          <t>COMPLEJO EDUCACIONAL CONSOLIDADA</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>COR. PUENTE</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>RIEGO</t>
+          <t>ESCUELA ANDES DEL SUR</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3643,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>COMPLEJO EDUCACIONAL CONSOLIDADA</t>
+          <t>ESCUELA GABRIELA</t>
         </is>
       </c>
     </row>
@@ -3655,7 +3655,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ESCUELA ANDES DEL SUR</t>
+          <t>ESCUELA JUAN MACKENNA</t>
         </is>
       </c>
     </row>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ESCUELA GABRIELA</t>
+          <t>ESCUELA LOS ANDES</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ESCUELA JUAN MACKENNA</t>
+          <t>ESCUELA LUIS MATTE LARRAIN</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ESCUELA LOS ANDES</t>
+          <t>ESCUELA PADRE HURTADO</t>
         </is>
       </c>
     </row>
@@ -3703,7 +3703,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ESCUELA LUIS MATTE LARRAIN</t>
+          <t>ESCUELA VILLA INDEPENDENCIA</t>
         </is>
       </c>
     </row>
@@ -3715,7 +3715,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ESCUELA PADRE HURTADO</t>
+          <t>ESCULA NONATO COO</t>
         </is>
       </c>
     </row>
@@ -3727,7 +3727,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ESCUELA VILLA INDEPENDENCIA</t>
+          <t>LICEO CHILOE</t>
         </is>
       </c>
     </row>
@@ -3739,31 +3739,31 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ESCULA NONATO COO</t>
+          <t>LICEO MAIPO</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LICEO CHILOE</t>
+          <t>ALICURA</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>COR. PUENTE</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LICEO MAIPO</t>
+          <t>ANTONIO HERMIDA FABRES</t>
         </is>
       </c>
     </row>
@@ -3775,7 +3775,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ALICURA</t>
+          <t>CARLOS FERNANDEZ PEÑA</t>
         </is>
       </c>
     </row>
@@ -3787,7 +3787,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ANTONIO HERMIDA FABRES</t>
+          <t>CENTRO EDUCACIONAL EDUARDO DE LA BARRA</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>CARLOS FERNANDEZ PEÑA</t>
+          <t>CENTRO EDUCACIONAL VALLE HERMOSO</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CENTRO EDUCACIONAL EDUARDO DE LA BARRA</t>
+          <t>ERASMO ESCALA</t>
         </is>
       </c>
     </row>
@@ -3823,7 +3823,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>CENTRO EDUCACIONAL VALLE HERMOSO</t>
+          <t>ESCUELA ESPECIAL PONTÍFICE JUAN PABLO II</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3835,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ERASMO ESCALA</t>
+          <t>ESCUELA LUIS ARRIETA CAÑAS</t>
         </is>
       </c>
     </row>
@@ -3847,7 +3847,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ESCUELA ESPECIAL PONTÍFICE JUAN PABLO II</t>
+          <t>ESCUELA UNIÓN NACIONAL ÁRABE</t>
         </is>
       </c>
     </row>
@@ -3859,7 +3859,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ESCUELA LUIS ARRIETA CAÑAS</t>
+          <t>JUAN BAUTISTA PASTENE</t>
         </is>
       </c>
     </row>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ESCUELA UNIÓN NACIONAL ÁRABE</t>
+          <t>LIKANKURA</t>
         </is>
       </c>
     </row>
@@ -3883,7 +3883,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>JUAN BAUTISTA PASTENE</t>
+          <t>MATILDE HUICI NAVAS</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>LIKANKURA</t>
+          <t>SANTA MARIA</t>
         </is>
       </c>
     </row>
@@ -3907,55 +3907,55 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>MATILDE HUICI NAVAS</t>
+          <t>TOBALABA</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>CUR</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>SANTA MARIA</t>
+          <t>ANILLO NORTE</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" t="inlineStr">
         <is>
-          <t>CORMUP</t>
+          <t>CUR</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>TOBALABA</t>
+          <t>ANILLO SUR</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="B58" t="inlineStr">
         <is>
-          <t>CUR</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ANILLO NORTE</t>
+          <t>QUILICURA - CAMARINES</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" t="inlineStr">
         <is>
-          <t>CUR</t>
+          <t>DERCO</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ANILLO SUR</t>
+          <t>QUILICURA - CASINO</t>
         </is>
       </c>
     </row>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>LO BOZA - EDIFICIO PRINCIPAL CASINO</t>
+          <t>QUILICURA - DERCOMAQ</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>LO BOZA - LAVADO DE VEHICULOS</t>
+          <t>QUILICURA - EDIFICIO JCB</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>LO BOZA - POZO DE LAVADO DE VEHICULO</t>
+          <t>QUILICURA - LAVADO DE MAQUINA</t>
         </is>
       </c>
     </row>
@@ -4003,7 +4003,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>LO BOZA - REUTILIZACION</t>
+          <t>QUILICURA - MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
@@ -4015,247 +4015,247 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>LO BOZA - SALA DE IMPULSION</t>
+          <t>QUILICURA - PRODERCO</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="B65" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>ESTADIO ISRAELITA</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>OPEN PLAZA - MATRIZ PRINCIPAL</t>
+          <t>MATRIS CHESTERTON</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="B66" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>ESTADIO ISRAELITA</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>PRONTO BAÑO</t>
+          <t>MATRIZ AV LAS CONDES</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="B67" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>QUILICURA - CAMARINES</t>
+          <t>ESTANQUE INFERIOR</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="B68" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>QUILICURA - CASINO</t>
+          <t>ETAPA 1</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="B69" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>QUILICURA - DERCOMAQ</t>
+          <t>ETAPA 1,2,3 Y 4</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="B70" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>QUILICURA - EDIFICIO JCB</t>
+          <t>ETAPA 1-4</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="B71" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>QUILICURA - LAVADO DE MAQUINA</t>
+          <t>ETAPA 2</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="B72" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>QUILICURA - MATRIZ PRINCIPAL</t>
+          <t>ETAPA 3</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="B73" t="inlineStr">
         <is>
-          <t>DERCO</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>QUILICURA - PRODERCO</t>
+          <t>ETAPA 5</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="B74" t="inlineStr">
         <is>
-          <t>ESTADIO ISRAELITA</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>MATRIS CHESTERTON</t>
+          <t>MATRIZ ESVAL</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="B75" t="inlineStr">
         <is>
-          <t>ESTADIO ISRAELITA</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>MATRIZ AV LAS CONDES</t>
+          <t>RIEGO LLENADO DE ESTANQUE ESVAL</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="B76" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ESTANQUE INFERIOR</t>
+          <t>CDP PUENTE ALTO</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="B77" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ETAPA 1</t>
+          <t>COLINA 1</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="B78" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ETAPA 1,2,3 Y 4</t>
+          <t>COLINA 2 RED SUR</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="B79" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>ETAPA 1-4</t>
+          <t>COLINA 2 REDIMPULSION</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="B80" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>ETAPA 2</t>
+          <t>CPA MODULO</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="B81" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ETAPA 3</t>
+          <t>CPA OVALO</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="B82" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ETAPA 5</t>
+          <t>CPF SAN MIGUEL MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="B83" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>MATRIS ESVAL</t>
+          <t>CPF SAN MIGUEL SALA IMPULSION</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="B84" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>GENCHI</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>RIEGO LLENADO DE ESTANQUE ESVAL</t>
+          <t>ESC. EL BOSQUE ADMINISTRACION</t>
         </is>
       </c>
     </row>
@@ -4267,7 +4267,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>CDP PUENTE ALTO</t>
+          <t>ESC. EL BOSQUE GENCHI ACADEMIA</t>
         </is>
       </c>
     </row>
@@ -4279,7 +4279,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>COLINA 1</t>
+          <t>ESC. OF ARTEMIO</t>
         </is>
       </c>
     </row>
@@ -4291,7 +4291,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>COLINA 2 RED SUR</t>
+          <t>ESC. OF CARMEN</t>
         </is>
       </c>
     </row>
@@ -4303,7 +4303,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>COLINA 2 REDIMPULSION</t>
+          <t>ESCUELA ANDES DEL SUR</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4315,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>CPA MODULO</t>
+          <t>ESFORPEN BOSQUE ADMINISTRACION</t>
         </is>
       </c>
     </row>
@@ -4327,7 +4327,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>CPA OVALO</t>
+          <t>ESFORPEN BOSQUE GENCHI SIMULACION</t>
         </is>
       </c>
     </row>
@@ -4339,7 +4339,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>CPF SAN MIGUEL MATRIZ PRINCIPAL</t>
+          <t>MONITOREO MATRIZ PRINCIPAL MODULO</t>
         </is>
       </c>
     </row>
@@ -4351,965 +4351,773 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>CPF SAN MIGUEL SALA IMPULSION</t>
+          <t>MONITOREO MATRIZ PRINCIPAL OVALO</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="B93" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>ESC. EL BOSQUE ADMINISTRACION</t>
+          <t>AGUA BLANDA</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="B94" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>ESC. EL BOSQUE GENCHI ACADEMIA</t>
+          <t>INTERCAMBIADOR 1</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="B95" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>ESC. OF ARTEMIO</t>
+          <t>INTERCAMBIADOR 2</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="B96" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>ESC. OF CARMEN</t>
+          <t>MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="B97" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>ESCUELA ANDES DEL SUR</t>
+          <t>RETORNO OSMOSIS</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="B98" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>HEGC</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>ESFORPEN BOSQUE ADMINISTRACION</t>
+          <t>SALIDA OSMOSIS</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="B99" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>LA FLORIDA</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>ESFORPEN BOSQUE GENCHI SIMULACION</t>
+          <t>LICEO ALTO CORDILLERA</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="B100" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>LA REINA</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>MONITOREO MATRIZ PRINCIPAL MODULO</t>
+          <t>EUGENIO MARIA DE HOSTOS</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="B101" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>LAS CONDES</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>MONITOREO MATRIZ PRINCIPAL OVALO</t>
+          <t>FLEMING</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>LO VALLEDOR</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>AGUA BLANDA</t>
+          <t>BARRIO NORTE</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="B103" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>LO VALLEDOR</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>INTERCAMBIADOR 1</t>
+          <t>POZO 1</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>LO VALLEDOR</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>INTERCAMBIADOR 2</t>
+          <t>PUERTA 1</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="B105" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>CASINO</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="B106" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>RETORNO OSMOSIS</t>
+          <t>ESTANQUE CISTERNA</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="B107" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>SALIDA OSMOSIS</t>
+          <t>SAN NICOLAS</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="B108" t="inlineStr">
         <is>
-          <t>LA FLORIDA</t>
+          <t>MADECCO</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>LICEO ALTO CORDILLERA</t>
+          <t>URETA COX</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
-          <t>LA REINA</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>EUGENIO MARIA DE HOSTOS</t>
+          <t>BAÑO GUARDIAS</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="B110" t="inlineStr">
         <is>
-          <t>LAS CONDES</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>FLEMING</t>
+          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="B111" t="inlineStr">
         <is>
-          <t>LAS CONDES</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>JUAN PABLO II</t>
+          <t>ESTANQUE NORTE LOCALES</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="B112" t="inlineStr">
         <is>
-          <t>LAS CONDES</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>LIKANKURA</t>
+          <t>PIZZA HUT</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="B113" t="inlineStr">
         <is>
-          <t>LO VALLEDOR</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>BARRIO NORTE</t>
+          <t>SALA DE BOMBAS ESTANQUE SUR</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="B114" t="inlineStr">
         <is>
-          <t>LO VALLEDOR</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>POZO 1</t>
+          <t>MATRIZ BOULEVARD PASILLO TECNICO</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="B115" t="inlineStr">
         <is>
-          <t>LO VALLEDOR</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>PUERTA 1</t>
+          <t>MATRIZ SALIDA DE EMERGENCIA PASILLO N°1 ARROW</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="B116" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>CASINO</t>
+          <t>PLACA BANCARIA</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="B117" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ESTANQUE CISTERNA</t>
+          <t>SALA DE BOMBAS FALABELLA</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="B118" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>SAN NICOLAS</t>
+          <t>SALA DE BOMBAS RIPLEY</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="B119" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>MAQ</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>URETA COX</t>
+          <t>ALIMENTACION DE BAÑOS</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="B120" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>MAQ</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>BAÑO GUARDIAS</t>
+          <t>MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="B121" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>MAQ</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
+          <t>RED DE INCENDIO</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="B122" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>MOLYMET</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>ESTANQUE NORTE LOCALES</t>
+          <t>CASA DE CAMBIO</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="B123" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>MOLYMET</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>KFC</t>
+          <t>RIEGO</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="B124" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>PIZZA HUT</t>
+          <t>CONTROL NIDO</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="B125" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS ESTANQUE SUR</t>
+          <t>ELEMENTARY</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="B126" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>MATRIZ BOULEVARD PASILLO TECNICO</t>
+          <t>ESTANQUE B</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="B127" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>MATRIZ SALIDA DE EMERGENCIA PASILLO N°1 ARROW</t>
+          <t>ESTANQUE C</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="B128" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>PLACA BANCARIA</t>
+          <t>HIGH SCHOOL</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="B129" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS FALABELLA</t>
+          <t>PISCINA</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="B130" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS RIPLEY</t>
+          <t>POZO PROFUNDO</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="B131" t="inlineStr">
         <is>
-          <t>MAQ</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ALIMENTACION DE BAÑOS</t>
+          <t>TEATRO</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="B132" t="inlineStr">
         <is>
-          <t>MAQ</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="B133" t="inlineStr">
         <is>
-          <t>MAQ</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>RED DE INCENDIO</t>
+          <t>ESTANQUE NORTE LOCALES</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="B134" t="inlineStr">
         <is>
-          <t>MOLYMET</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>CASA DE CAMBIO</t>
+          <t>KFC</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="B135" t="inlineStr">
         <is>
-          <t>MOLYMET</t>
+          <t>PAE</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>RIEGO</t>
+          <t>PIZZA HUT</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="B136" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>CANCHA</t>
+          <t>ANDEN 3-4 LOCALES GASTRONOMICOS</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="B137" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>CONTROL NIDO</t>
+          <t>ANDEN 3-4 MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="B138" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>ELEMENTARY</t>
+          <t>ANDEN 3-4 RESTAURANTE</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="B139" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ESTANQUE B</t>
+          <t>BAZAR GOURMET</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="B140" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ESTANQUE C</t>
+          <t>DISTRITO DE LUJO</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="B141" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>HIGH SCHOOL</t>
+          <t>DL KENNEDY</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="B142" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>PISCINA</t>
+          <t>LLENADO DE PILETA</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="B143" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>POZO PROFUNDO</t>
+          <t>PILETA CASCADA</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="B144" t="inlineStr">
         <is>
-          <t>NIDO</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>TEATRO</t>
+          <t>SANDIA ANTIGUA</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="B145" t="inlineStr">
         <is>
-          <t>PAE</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
+          <t>SANDIA NUEVA</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="B146" t="inlineStr">
         <is>
-          <t>PAE</t>
+          <t>PROVIDENCIA</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>ESTANQUE NORTE LOCALES</t>
+          <t>CARMELA CARVAJAL</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="B147" t="inlineStr">
         <is>
-          <t>PAE</t>
+          <t>PROVIDENCIA</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>KFC</t>
+          <t>LASTARRIA</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="B148" t="inlineStr">
         <is>
-          <t>PAE</t>
+          <t>PROVIDENCIA</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>PIZZA HUT</t>
+          <t>LICEO JUAN PABLO DUARTE</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="B149" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>PROVIDENCIA</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>ANDEN 3-4 LOCALES GASTRONOMICOS</t>
+          <t>LICEO N°7</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="B150" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>RENCA</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>ANDEN 3-4 MATRIZ PRINCIPAL</t>
+          <t>ESCUELA LO VELEZQUEZ</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="B151" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>RENCA</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>ANDEN 3-4 RESTAURANTE</t>
+          <t>GIMNASIO MUNICIPAL</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="B152" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>RENCA</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>BAZAR GOURMET</t>
+          <t>ICCO</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="B153" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>RENCA</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>DISTRITO DE LUJO</t>
+          <t>ICCP</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="B154" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>RENCA</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>DL KENNEDY</t>
+          <t>PISCINA MUNICIPAL</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="B155" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>UDD</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>LLENADO DE PILETA</t>
+          <t>SALA DE BOMBAS EDIFICIO ¨O¨</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="B156" t="inlineStr">
         <is>
-          <t>PAK</t>
+          <t>UDD</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
-        <is>
-          <t>PILETA CASCADA</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>PAK</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>SANDIA ANTIGUA</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>PAK</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>SANDIA NUEVA</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>PROVIDENCIA</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>CARMELA CARVAJAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>PROVIDENCIA</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>LASTARRIA</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>PROVIDENCIA</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>LICEO JUAN PABLO DUARTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>PROVIDENCIA</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>LICEO N°7</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>RENCA</t>
-        </is>
-      </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>CAPITAN JOSÉ LUIS ARANDE</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>RENCA</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>ESCUELA LO VELZAQUEZ</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>RENCA</t>
-        </is>
-      </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>GYM MUNICIPAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>RENCA</t>
-        </is>
-      </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>INSTITUTO CUMBRE DE CONDORES ORIENTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>RENCA</t>
-        </is>
-      </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>INSTITUTO CUMBRE DE CONDORES PONIENTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>RENCA</t>
-        </is>
-      </c>
-      <c r="C168" t="inlineStr">
-        <is>
-          <t>JUAN DE ATALA HIRMAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>RENCA</t>
-        </is>
-      </c>
-      <c r="C169" t="inlineStr">
-        <is>
-          <t>PISCINA MUNICIPAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>RENCA</t>
-        </is>
-      </c>
-      <c r="C170" t="inlineStr">
-        <is>
-          <t>REBECA MATTE BELLO</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>UDD</t>
-        </is>
-      </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>SALA DE BOMBAS EDIFICIO ¨O¨</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>UDD</t>
-        </is>
-      </c>
-      <c r="C172" t="inlineStr">
         <is>
           <t>SALA DE BOMBAS HONDURAS</t>
         </is>
@@ -5335,7 +5143,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="20">
-        <f>IFERROR(FILTER(Base1!B2:C172,Base1!B2:B172=Ingreso!C4),"")</f>
+        <f>IFERROR(FILTER(Base1!B2:C156,Base1!B2:B156=Ingreso!C4),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>